<commit_message>
update qrevo videos + report (2026-07-05 10:07 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,45 +517,45 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>phanthulan715</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>684</v>
+        <v>857</v>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.63</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>phanthulan715</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>731</v>
+        <v>684</v>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>3.15</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="7">
@@ -583,190 +583,190 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>488</v>
+        <v>1097</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>5.12</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>432</v>
+        <v>488</v>
       </c>
       <c r="D9" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
-        <v>21.53</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>629</v>
+        <v>471</v>
       </c>
       <c r="D10" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>7.63</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>466</v>
+        <v>432</v>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F11" t="n">
-        <v>3.86</v>
+        <v>21.53</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>389</v>
+        <v>241</v>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>2.57</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>271</v>
+        <v>629</v>
       </c>
       <c r="D13" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="F13" t="n">
-        <v>5.54</v>
+        <v>7.63</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>23</v>
+        <v>389</v>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>26.09</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>332</v>
+        <v>271</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>2.11</v>
+        <v>5.54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>229</v>
+        <v>23</v>
       </c>
       <c r="D16" t="n">
         <v>6</v>
@@ -775,152 +775,152 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>2.62</v>
+        <v>26.09</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>208</v>
+        <v>332</v>
       </c>
       <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="n">
         <v>1</v>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
       <c r="F17" t="n">
-        <v>0.48</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>2</v>
       </c>
       <c r="C18" t="n">
+        <v>229</v>
+      </c>
+      <c r="D18" t="n">
         <v>6</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>208</v>
+      </c>
+      <c r="D19" t="n">
         <v>1</v>
       </c>
-      <c r="C19" t="n">
-        <v>358</v>
-      </c>
-      <c r="D19" t="n">
-        <v>7</v>
-      </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>2.51</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>1.44</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>241</v>
+        <v>347</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>1.24</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>177</v>
+        <v>241</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2.82</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>131</v>
+        <v>177</v>
       </c>
       <c r="D23" t="n">
         <v>5</v>
@@ -929,50 +929,72 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>3.82</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>3.08</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>tm.anh.kitchen.qu</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>130</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>93</v>
-      </c>
-      <c r="C25" t="n">
-        <v>17499</v>
-      </c>
-      <c r="D25" t="n">
-        <v>468</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="B26" t="n">
+        <v>103</v>
+      </c>
+      <c r="C26" t="n">
+        <v>18962</v>
+      </c>
+      <c r="D26" t="n">
+        <v>478</v>
+      </c>
+      <c r="E26" t="n">
         <v>124</v>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-05 12:02 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="D7" t="n">
         <v>6</v>
@@ -577,7 +577,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="8">
@@ -587,107 +587,107 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>1097</v>
+        <v>1112</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.46</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>488</v>
+        <v>284</v>
       </c>
       <c r="D9" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>5.12</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>471</v>
+        <v>488</v>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
-        <v>3.82</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>432</v>
+        <v>471</v>
       </c>
       <c r="D11" t="n">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E11" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>21.53</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>241</v>
+        <v>432</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>0.41</v>
+        <v>21.53</v>
       </c>
     </row>
     <row r="13">
@@ -983,13 +983,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C26" t="n">
-        <v>18962</v>
+        <v>19027</v>
       </c>
       <c r="D26" t="n">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E26" t="n">
         <v>124</v>

</xml_diff>

<commit_message>
data: realtime crawl 05/07 23:44 VN (114 videos, +8); remove stale pptx snapshot
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,151 +477,151 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>2666</v>
+        <v>3321</v>
       </c>
       <c r="D3" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>2.14</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>5953</v>
+        <v>481</v>
       </c>
       <c r="D4" t="n">
-        <v>105</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1.81</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>phanthulan715</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>857</v>
+        <v>5953</v>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>3.15</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>phanthulan715</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>684</v>
+        <v>857</v>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2.63</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1.02</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>1112</v>
+        <v>685</v>
       </c>
       <c r="D8" t="n">
         <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.54</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>284</v>
+        <v>1112</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="10">
@@ -781,133 +781,133 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>2.11</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>229</v>
+        <v>332</v>
       </c>
       <c r="D18" t="n">
         <v>6</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2.62</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.48</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>208</v>
+      </c>
+      <c r="D20" t="n">
         <v>1</v>
       </c>
-      <c r="C20" t="n">
-        <v>358</v>
-      </c>
-      <c r="D20" t="n">
-        <v>7</v>
-      </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>2.51</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>1.44</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>241</v>
+        <v>347</v>
       </c>
       <c r="D22" t="n">
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>1.24</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="23">
@@ -983,16 +983,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C26" t="n">
-        <v>19027</v>
+        <v>19985</v>
       </c>
       <c r="D26" t="n">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="E26" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F26" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
data: crawl 06/07 13:12 VN (124 videos, +10); pending dealers 20->19
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,151 +477,151 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>3321</v>
+        <v>3361</v>
       </c>
       <c r="D3" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>1.84</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>481</v>
+        <v>703</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.83</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>5953</v>
+        <v>481</v>
       </c>
       <c r="D5" t="n">
-        <v>105</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1.81</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>phanthulan715</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>857</v>
+        <v>1213</v>
       </c>
       <c r="D6" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>3.15</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>684</v>
+        <v>5953</v>
       </c>
       <c r="D7" t="n">
-        <v>18</v>
+        <v>105</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>2.63</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>phanthulan715</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C8" t="n">
-        <v>685</v>
+        <v>857</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1.02</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>1112</v>
+        <v>685</v>
       </c>
       <c r="D9" t="n">
         <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.54</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="10">
@@ -781,168 +781,168 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>347</v>
+        <v>2199</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>1.15</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>2.11</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>229</v>
+        <v>332</v>
       </c>
       <c r="D19" t="n">
         <v>6</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.62</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.48</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>208</v>
+      </c>
+      <c r="D21" t="n">
         <v>1</v>
       </c>
-      <c r="C21" t="n">
-        <v>358</v>
-      </c>
-      <c r="D21" t="n">
-        <v>7</v>
-      </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.51</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>1.44</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>177</v>
+        <v>347</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>2.82</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>131</v>
+        <v>177</v>
       </c>
       <c r="D24" t="n">
         <v>5</v>
@@ -951,50 +951,94 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>3.82</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>3.08</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>tm.anh.kitchen.qu</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>130</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>anhlinhgroup_73</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>15</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>114</v>
-      </c>
-      <c r="C26" t="n">
-        <v>19985</v>
-      </c>
-      <c r="D26" t="n">
-        <v>486</v>
-      </c>
-      <c r="E26" t="n">
-        <v>125</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="B28" t="n">
+        <v>124</v>
+      </c>
+      <c r="C28" t="n">
+        <v>22359</v>
+      </c>
+      <c r="D28" t="n">
+        <v>525</v>
+      </c>
+      <c r="E28" t="n">
+        <v>143</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: auto-refresh view/like/comment for videos within 21-day window
Fixes frozen metrics — the crawler captured each video once at post time
(near-zero views) and never updated it. Total views corrected 22k -> 90k
after refreshing 118 recent videos.
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,16 +458,16 @@
         <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>1930</v>
+        <v>2299</v>
       </c>
       <c r="D2" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="E2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F2" t="n">
-        <v>6.17</v>
+        <v>6.39</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>3361</v>
+        <v>62707</v>
       </c>
       <c r="D3" t="n">
-        <v>53</v>
+        <v>289</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="F3" t="n">
-        <v>1.87</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>703</v>
+        <v>1501</v>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2.7</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>481</v>
+        <v>1148</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>1213</v>
+        <v>2071</v>
       </c>
       <c r="D6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E6" t="n">
         <v>10</v>
       </c>
-      <c r="E6" t="n">
-        <v>3</v>
-      </c>
       <c r="F6" t="n">
-        <v>1.07</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>5953</v>
+        <v>6104</v>
       </c>
       <c r="D7" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>1.81</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="8">
@@ -590,16 +590,16 @@
         <v>9</v>
       </c>
       <c r="C8" t="n">
-        <v>857</v>
+        <v>1686</v>
       </c>
       <c r="D8" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>3.15</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="9">
@@ -612,82 +612,82 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>685</v>
+        <v>944</v>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>1.02</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>488</v>
+        <v>693</v>
       </c>
       <c r="D10" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5.12</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>471</v>
+        <v>641</v>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="F11" t="n">
-        <v>3.82</v>
+        <v>19.19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>432</v>
+        <v>519</v>
       </c>
       <c r="D12" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>21.53</v>
+        <v>5.01</v>
       </c>
     </row>
     <row r="13">
@@ -700,60 +700,60 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>629</v>
+        <v>1153</v>
       </c>
       <c r="D13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" t="n">
         <v>26</v>
       </c>
-      <c r="E13" t="n">
-        <v>22</v>
-      </c>
       <c r="F13" t="n">
-        <v>7.63</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>389</v>
+        <v>1095</v>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>2.57</v>
+        <v>7.03</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>271</v>
+        <v>482</v>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
         <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>5.54</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="16">
@@ -766,16 +766,16 @@
         <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>26.09</v>
+        <v>25.93</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>2199</v>
+        <v>2234</v>
       </c>
       <c r="D17" t="n">
         <v>32</v>
@@ -797,7 +797,7 @@
         <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>2.14</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="18">
@@ -810,104 +810,104 @@
         <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>347</v>
+        <v>1197</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>259</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
-        <v>1.15</v>
+        <v>22.31</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>332</v>
+        <v>788</v>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.11</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>229</v>
+        <v>376</v>
       </c>
       <c r="D20" t="n">
         <v>6</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2.62</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>208</v>
+        <v>305</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.48</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>358</v>
+        <v>1082</v>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2.51</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="23">
@@ -920,82 +920,82 @@
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>347</v>
+        <v>427</v>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>1.44</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>177</v>
+        <v>358</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>2.82</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>131</v>
+        <v>214</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>3.82</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>130</v>
+        <v>179</v>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>3.08</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1030,13 +1030,13 @@
         <v>124</v>
       </c>
       <c r="C28" t="n">
-        <v>22359</v>
+        <v>90315</v>
       </c>
       <c r="D28" t="n">
-        <v>525</v>
+        <v>1227</v>
       </c>
       <c r="E28" t="n">
-        <v>143</v>
+        <v>258</v>
       </c>
       <c r="F28" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-06 14:31 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>2299</v>
+        <v>2371</v>
       </c>
       <c r="D2" t="n">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="E2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F2" t="n">
-        <v>6.39</v>
+        <v>6.96</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>62707</v>
+        <v>68696</v>
       </c>
       <c r="D3" t="n">
-        <v>289</v>
+        <v>307</v>
       </c>
       <c r="E3" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F3" t="n">
-        <v>0.59</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="4">
@@ -499,173 +499,173 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>1501</v>
+        <v>1848</v>
       </c>
       <c r="D4" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2.27</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>1148</v>
+        <v>2536</v>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>0.78</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>phanthulan715</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>2071</v>
+        <v>1958</v>
       </c>
       <c r="D6" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2.27</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1170</v>
+      </c>
+      <c r="D7" t="n">
         <v>9</v>
       </c>
-      <c r="C7" t="n">
-        <v>6104</v>
-      </c>
-      <c r="D7" t="n">
-        <v>107</v>
-      </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1.82</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>phanthulan715</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1686</v>
+        <v>1167</v>
       </c>
       <c r="D8" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>2.43</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>944</v>
+        <v>6139</v>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>1.38</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>693</v>
+        <v>1069</v>
       </c>
       <c r="D10" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>3.9</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C11" t="n">
-        <v>641</v>
+        <v>1111</v>
       </c>
       <c r="D11" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="E11" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>19.19</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="12">
@@ -675,370 +675,458 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="D12" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" t="n">
         <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>5.01</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>1153</v>
+        <v>699</v>
       </c>
       <c r="D13" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="E13" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>5.29</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>1095</v>
+        <v>649</v>
       </c>
       <c r="D14" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="F14" t="n">
-        <v>7.03</v>
+        <v>19.26</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>482</v>
+        <v>407</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>2.49</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>27</v>
+        <v>1162</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F16" t="n">
-        <v>25.93</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>2234</v>
+        <v>1109</v>
       </c>
       <c r="D17" t="n">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F17" t="n">
-        <v>2.1</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>1197</v>
+        <v>486</v>
       </c>
       <c r="D18" t="n">
-        <v>259</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>22.31</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>788</v>
+        <v>401</v>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>1.52</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>376</v>
+        <v>29</v>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>1.86</v>
+        <v>24.14</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>305</v>
+        <v>2290</v>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F21" t="n">
-        <v>2.3</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>1082</v>
+        <v>1775</v>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>554</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F22" t="n">
-        <v>1.02</v>
+        <v>31.94</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>427</v>
+        <v>788</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1.41</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>358</v>
+        <v>376</v>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2.51</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>214</v>
+        <v>1451</v>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>3.74</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>179</v>
+        <v>1085</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>2.79</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>85</v>
+        <v>435</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>caothienphat.official</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>358</v>
+      </c>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>tm.anh.kitchen.qu</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>216</v>
+      </c>
+      <c r="D29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>anhlinhgroup_73</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>100</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>bepphuthai</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>22</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>124</v>
-      </c>
-      <c r="C28" t="n">
-        <v>90315</v>
-      </c>
-      <c r="D28" t="n">
-        <v>1227</v>
-      </c>
-      <c r="E28" t="n">
-        <v>258</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="B32" t="n">
+        <v>155</v>
+      </c>
+      <c r="C32" t="n">
+        <v>102444</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1627</v>
+      </c>
+      <c r="E32" t="n">
+        <v>276</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: crawl 07/07 11:08 VN (162 videos, +38); refresh views -> 220k; 31 dealers
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,148 +458,148 @@
         <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>2371</v>
+        <v>2438</v>
       </c>
       <c r="D2" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E2" t="n">
         <v>26</v>
       </c>
       <c r="F2" t="n">
-        <v>6.96</v>
+        <v>6.93</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>phanthulan715</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>68696</v>
+        <v>2329</v>
       </c>
       <c r="D3" t="n">
-        <v>307</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>83</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>0.57</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>1848</v>
+        <v>183780</v>
       </c>
       <c r="D4" t="n">
-        <v>44</v>
+        <v>1000</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>209</v>
       </c>
       <c r="F4" t="n">
-        <v>2.38</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>2536</v>
+        <v>1895</v>
       </c>
       <c r="D5" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.25</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>phanthulan715</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>1958</v>
+        <v>2936</v>
       </c>
       <c r="D6" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>2.3</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>1170</v>
+        <v>1312</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.77</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1167</v>
+        <v>1203</v>
       </c>
       <c r="D8" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1.71</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="9">
@@ -612,16 +612,16 @@
         <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>6139</v>
+        <v>6153</v>
       </c>
       <c r="D9" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E9" t="n">
         <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>1.82</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="10">
@@ -634,16 +634,16 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>1069</v>
+        <v>1081</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>1.5</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="11">
@@ -656,7 +656,7 @@
         <v>6</v>
       </c>
       <c r="C11" t="n">
-        <v>1111</v>
+        <v>1134</v>
       </c>
       <c r="D11" t="n">
         <v>16</v>
@@ -665,7 +665,7 @@
         <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>1.62</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="12">
@@ -678,16 +678,16 @@
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>541</v>
+        <v>629</v>
       </c>
       <c r="D12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E12" t="n">
         <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>4.99</v>
+        <v>4.61</v>
       </c>
     </row>
     <row r="13">
@@ -700,16 +700,16 @@
         <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>699</v>
+        <v>713</v>
       </c>
       <c r="D13" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3.86</v>
+        <v>3.93</v>
       </c>
     </row>
     <row r="14">
@@ -722,16 +722,16 @@
         <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>649</v>
+        <v>662</v>
       </c>
       <c r="D14" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E14" t="n">
         <v>65</v>
       </c>
       <c r="F14" t="n">
-        <v>19.26</v>
+        <v>19.03</v>
       </c>
     </row>
     <row r="15">
@@ -744,16 +744,16 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>407</v>
+        <v>505</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>1.47</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>1162</v>
+        <v>1181</v>
       </c>
       <c r="D16" t="n">
         <v>35</v>
@@ -775,7 +775,7 @@
         <v>26</v>
       </c>
       <c r="F16" t="n">
-        <v>5.25</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="17">
@@ -788,16 +788,16 @@
         <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>1109</v>
+        <v>1124</v>
       </c>
       <c r="D17" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F17" t="n">
-        <v>7.57</v>
+        <v>7.74</v>
       </c>
     </row>
     <row r="18">
@@ -810,7 +810,7 @@
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="D18" t="n">
         <v>8</v>
@@ -819,7 +819,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>2.47</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="19">
@@ -832,301 +832,323 @@
         <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>401</v>
+        <v>440</v>
       </c>
       <c r="D19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>2.24</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>29</v>
+        <v>398</v>
       </c>
       <c r="D20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>24.14</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>2290</v>
+        <v>31</v>
       </c>
       <c r="D21" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.05</v>
+        <v>22.58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>1775</v>
+        <v>2435</v>
       </c>
       <c r="D22" t="n">
-        <v>554</v>
+        <v>33</v>
       </c>
       <c r="E22" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>31.94</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>788</v>
+        <v>1871</v>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>563</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>1.52</v>
+        <v>30.89</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>376</v>
+        <v>794</v>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>1.86</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>1451</v>
+        <v>379</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>1085</v>
+        <v>2590</v>
       </c>
       <c r="D26" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1.01</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>435</v>
+        <v>1120</v>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>1.38</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>358</v>
+        <v>454</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
         <v>2</v>
       </c>
       <c r="F28" t="n">
-        <v>2.51</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>216</v>
+        <v>358</v>
       </c>
       <c r="D29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>3.7</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>100</v>
+        <v>224</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>anhlinhgroup_73</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>22</v>
+        <v>117</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>bepphuthai</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>94</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2.13</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>155</v>
-      </c>
-      <c r="C32" t="n">
-        <v>102444</v>
-      </c>
-      <c r="D32" t="n">
-        <v>1627</v>
-      </c>
-      <c r="E32" t="n">
-        <v>276</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="B33" t="n">
+        <v>162</v>
+      </c>
+      <c r="C33" t="n">
+        <v>220872</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2377</v>
+      </c>
+      <c r="E33" t="n">
+        <v>408</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-07 13:07 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,45 +451,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>phanthulan715</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>2438</v>
+        <v>2482</v>
       </c>
       <c r="D2" t="n">
-        <v>143</v>
+        <v>58</v>
       </c>
       <c r="E2" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>6.93</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>phanthulan715</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>2329</v>
+        <v>2462</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>145</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>2.4</v>
+        <v>6.95</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>183780</v>
+        <v>274953</v>
       </c>
       <c r="D4" t="n">
-        <v>1000</v>
+        <v>1611</v>
       </c>
       <c r="E4" t="n">
-        <v>209</v>
+        <v>286</v>
       </c>
       <c r="F4" t="n">
-        <v>0.66</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -524,10 +524,10 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>1895</v>
+        <v>1944</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -546,7 +546,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>2936</v>
+        <v>3128</v>
       </c>
       <c r="D6" t="n">
         <v>51</v>
@@ -555,7 +555,7 @@
         <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>2.11</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>1312</v>
+        <v>1385</v>
       </c>
       <c r="D7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1.75</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="8">
@@ -590,7 +590,7 @@
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1203</v>
+        <v>1208</v>
       </c>
       <c r="D8" t="n">
         <v>9</v>
@@ -609,546 +609,612 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>6153</v>
+        <v>6446</v>
       </c>
       <c r="D9" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E9" t="n">
         <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>1.84</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>1081</v>
+        <v>920</v>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="F10" t="n">
-        <v>1.67</v>
+        <v>15.65</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>1134</v>
+        <v>1083</v>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>1.59</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>629</v>
+        <v>1137</v>
       </c>
       <c r="D12" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>4.61</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>713</v>
+        <v>1296</v>
       </c>
       <c r="D13" t="n">
+        <v>38</v>
+      </c>
+      <c r="E13" t="n">
         <v>27</v>
       </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" t="n">
-        <v>3.93</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>662</v>
+        <v>697</v>
       </c>
       <c r="D14" t="n">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="E14" t="n">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>19.03</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>505</v>
+        <v>726</v>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>2.18</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>1181</v>
+        <v>518</v>
       </c>
       <c r="D16" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>5.17</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>1124</v>
+        <v>435</v>
       </c>
       <c r="D17" t="n">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>7.74</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>492</v>
+        <v>1160</v>
       </c>
       <c r="D18" t="n">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F18" t="n">
-        <v>2.44</v>
+        <v>7.67</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>440</v>
+        <v>877</v>
       </c>
       <c r="D19" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>2.27</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>398</v>
+        <v>698</v>
       </c>
       <c r="D20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>2.26</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>31</v>
+        <v>497</v>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>22.58</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>2435</v>
+        <v>493</v>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="E22" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>1.97</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>1871</v>
+        <v>454</v>
       </c>
       <c r="D23" t="n">
-        <v>563</v>
+        <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>30.89</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>794</v>
+        <v>40</v>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>1.51</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>379</v>
+        <v>2491</v>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F25" t="n">
-        <v>1.06</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2590</v>
+        <v>2021</v>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>563</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F26" t="n">
-        <v>0.15</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>1120</v>
+        <v>796</v>
       </c>
       <c r="D27" t="n">
         <v>11</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>0.98</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>454</v>
+        <v>629</v>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>1.32</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>ecomi.vn.roborock</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>358</v>
+        <v>176</v>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.51</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>224</v>
+        <v>2591</v>
       </c>
       <c r="D30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>3.57</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>117</v>
+        <v>1145</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0.85</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>94</v>
+        <v>468</v>
       </c>
       <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="n">
         <v>2</v>
       </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
       <c r="F32" t="n">
-        <v>2.13</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>caothienphat.official</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>358</v>
+      </c>
+      <c r="D33" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>anhlinhgroup_73</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>118</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>bepphuthai</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>117</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>162</v>
-      </c>
-      <c r="C33" t="n">
-        <v>220872</v>
-      </c>
-      <c r="D33" t="n">
-        <v>2377</v>
-      </c>
-      <c r="E33" t="n">
-        <v>408</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="B36" t="n">
+        <v>182</v>
+      </c>
+      <c r="C36" t="n">
+        <v>315949</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3071</v>
+      </c>
+      <c r="E36" t="n">
+        <v>496</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: crawl 08/07 13:48 VN (191 videos, +10 vs 181); refresh views -> 404k; 36 dealers
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>2482</v>
+        <v>2985</v>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F2" t="n">
-        <v>2.42</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>2462</v>
+        <v>2542</v>
       </c>
       <c r="D3" t="n">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="E3" t="n">
         <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>6.95</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>274953</v>
+        <v>360342</v>
       </c>
       <c r="D4" t="n">
-        <v>1611</v>
+        <v>2154</v>
       </c>
       <c r="E4" t="n">
-        <v>286</v>
+        <v>369</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5">
@@ -524,126 +524,126 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>1944</v>
+        <v>1983</v>
       </c>
       <c r="D5" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.37</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>3128</v>
+        <v>1407</v>
       </c>
       <c r="D6" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="F6" t="n">
-        <v>1.98</v>
+        <v>10.66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>1385</v>
+        <v>3168</v>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>1.73</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1208</v>
+        <v>1435</v>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.75</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>6446</v>
+        <v>1217</v>
       </c>
       <c r="D9" t="n">
-        <v>115</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1.85</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>920</v>
+        <v>6563</v>
       </c>
       <c r="D10" t="n">
-        <v>72</v>
+        <v>120</v>
       </c>
       <c r="E10" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>15.65</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="11">
@@ -656,7 +656,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>1083</v>
+        <v>1091</v>
       </c>
       <c r="D11" t="n">
         <v>15</v>
@@ -665,7 +665,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>1.66</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="12">
@@ -678,16 +678,16 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>1137</v>
+        <v>1151</v>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>1.58</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="13">
@@ -700,16 +700,16 @@
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>1296</v>
+        <v>1491</v>
       </c>
       <c r="D13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E13" t="n">
         <v>27</v>
       </c>
       <c r="F13" t="n">
-        <v>5.02</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="14">
@@ -722,148 +722,148 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="D14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E14" t="n">
         <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>4.45</v>
+        <v>4.56</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>726</v>
+        <v>1195</v>
       </c>
       <c r="D15" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>3.86</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>518</v>
+        <v>734</v>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>2.12</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>435</v>
+        <v>521</v>
       </c>
       <c r="D17" t="n">
         <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>2.76</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1160</v>
+        <v>471</v>
       </c>
       <c r="D18" t="n">
-        <v>76</v>
+        <v>14</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>7.67</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>877</v>
+        <v>1186</v>
       </c>
       <c r="D19" t="n">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F19" t="n">
-        <v>2.39</v>
+        <v>7.59</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>698</v>
+        <v>1009</v>
       </c>
       <c r="D20" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>1.29</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="21">
@@ -876,16 +876,16 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>497</v>
+        <v>532</v>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.01</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D22" t="n">
         <v>8</v>
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D23" t="n">
         <v>10</v>
@@ -929,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D24" t="n">
         <v>9</v>
@@ -951,7 +951,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>22.5</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="25">
@@ -964,7 +964,7 @@
         <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>2491</v>
+        <v>2541</v>
       </c>
       <c r="D25" t="n">
         <v>33</v>
@@ -973,7 +973,7 @@
         <v>15</v>
       </c>
       <c r="F25" t="n">
-        <v>1.93</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="26">
@@ -986,16 +986,16 @@
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2021</v>
+        <v>2336</v>
       </c>
       <c r="D26" t="n">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="E26" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F26" t="n">
-        <v>28.6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="D27" t="n">
         <v>11</v>
@@ -1030,16 +1030,16 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>629</v>
+        <v>692</v>
       </c>
       <c r="D28" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.38</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>176</v>
+        <v>252</v>
       </c>
       <c r="D29" t="n">
         <v>4</v>
@@ -1061,7 +1061,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.27</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>2591</v>
+        <v>2592</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1096,16 +1096,16 @@
         <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>1145</v>
+        <v>1201</v>
       </c>
       <c r="D31" t="n">
         <v>12</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>1.05</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="32">
@@ -1118,7 +1118,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>468</v>
+        <v>490</v>
       </c>
       <c r="D32" t="n">
         <v>4</v>
@@ -1127,7 +1127,7 @@
         <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="33">
@@ -1155,14 +1155,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>roborock.smart.li</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>118</v>
+        <v>225</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0.85</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="35">
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1193,28 +1193,72 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>2.56</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>anhlinhgroup_73</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>118</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mistorebienhoa</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>11</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>182</v>
-      </c>
-      <c r="C36" t="n">
-        <v>315949</v>
-      </c>
-      <c r="D36" t="n">
-        <v>3071</v>
-      </c>
-      <c r="E36" t="n">
-        <v>496</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
+      <c r="B38" t="n">
+        <v>191</v>
+      </c>
+      <c r="C38" t="n">
+        <v>404450</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3717</v>
+      </c>
+      <c r="E38" t="n">
+        <v>604</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-08 12:26 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,16 +458,16 @@
         <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>2985</v>
+        <v>3074</v>
       </c>
       <c r="D2" t="n">
         <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" t="n">
-        <v>3.82</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="3">
@@ -480,7 +480,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>2542</v>
+        <v>2568</v>
       </c>
       <c r="D3" t="n">
         <v>170</v>
@@ -489,7 +489,7 @@
         <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>7.71</v>
+        <v>7.63</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>360342</v>
+        <v>384464</v>
       </c>
       <c r="D4" t="n">
-        <v>2154</v>
+        <v>2276</v>
       </c>
       <c r="E4" t="n">
-        <v>369</v>
+        <v>405</v>
       </c>
       <c r="F4" t="n">
         <v>0.7</v>
@@ -524,7 +524,7 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>1983</v>
+        <v>2011</v>
       </c>
       <c r="D5" t="n">
         <v>48</v>
@@ -533,7 +533,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.42</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="6">
@@ -543,107 +543,107 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>1407</v>
+        <v>1473</v>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E6" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>10.66</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>3168</v>
+        <v>1485</v>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>1.96</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1435</v>
+        <v>6936</v>
       </c>
       <c r="D8" t="n">
-        <v>25</v>
+        <v>131</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
-        <v>1.74</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>1217</v>
+        <v>3193</v>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>0.74</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C10" t="n">
-        <v>6563</v>
+        <v>1217</v>
       </c>
       <c r="D10" t="n">
-        <v>120</v>
+        <v>9</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1.89</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="11">
@@ -656,7 +656,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>1091</v>
+        <v>1096</v>
       </c>
       <c r="D11" t="n">
         <v>15</v>
@@ -665,7 +665,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>1.65</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="12">
@@ -678,7 +678,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>1151</v>
+        <v>1161</v>
       </c>
       <c r="D12" t="n">
         <v>17</v>
@@ -687,7 +687,7 @@
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>1.65</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="13">
@@ -700,16 +700,16 @@
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>1491</v>
+        <v>1517</v>
       </c>
       <c r="D13" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E13" t="n">
         <v>27</v>
       </c>
       <c r="F13" t="n">
-        <v>4.43</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="D14" t="n">
         <v>26</v>
@@ -731,7 +731,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>4.56</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>1195</v>
+        <v>1258</v>
       </c>
       <c r="D15" t="n">
         <v>18</v>
@@ -753,271 +753,271 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>1.51</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>734</v>
+        <v>1102</v>
       </c>
       <c r="D16" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>3.81</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>521</v>
+        <v>739</v>
       </c>
       <c r="D17" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2.11</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>471</v>
+        <v>522</v>
       </c>
       <c r="D18" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>3.4</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>1186</v>
+        <v>477</v>
       </c>
       <c r="D19" t="n">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="E19" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>7.59</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>1009</v>
+        <v>1195</v>
       </c>
       <c r="D20" t="n">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F20" t="n">
-        <v>2.38</v>
+        <v>7.62</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>532</v>
+        <v>823</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.26</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>494</v>
+        <v>535</v>
       </c>
       <c r="D22" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.43</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>457</v>
+        <v>496</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>2.19</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>43</v>
+        <v>461</v>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>20.93</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>2541</v>
+        <v>43</v>
       </c>
       <c r="D25" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>1.89</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2336</v>
+        <v>2552</v>
       </c>
       <c r="D26" t="n">
-        <v>566</v>
+        <v>33</v>
       </c>
       <c r="E26" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F26" t="n">
-        <v>25</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>797</v>
+        <v>2493</v>
       </c>
       <c r="D27" t="n">
-        <v>11</v>
+        <v>566</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F27" t="n">
-        <v>1.51</v>
+        <v>23.43</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="D28" t="n">
         <v>18</v>
@@ -1039,42 +1039,42 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.6</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ecomi.vn.roborock</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>252</v>
+        <v>419</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.59</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>ecomi.vn.roborock</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>2592</v>
+        <v>258</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1083,182 +1083,204 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.15</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>1201</v>
+        <v>159</v>
       </c>
       <c r="D31" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>490</v>
+        <v>2592</v>
       </c>
       <c r="D32" t="n">
         <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>1.22</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>358</v>
+        <v>1220</v>
       </c>
       <c r="D33" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>2.51</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>roborock.smart.li</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>225</v>
+        <v>501</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
-        <v>0.44</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>roborock.smart.li</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>119</v>
+        <v>319</v>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>2.52</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>bepphuthai</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.85</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>anhlinhgroup_73</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>11</v>
+        <v>118</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>mistorebienhoa</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>83</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2.41</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>191</v>
-      </c>
-      <c r="C38" t="n">
-        <v>404450</v>
-      </c>
-      <c r="D38" t="n">
-        <v>3717</v>
-      </c>
-      <c r="E38" t="n">
-        <v>604</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="B39" t="n">
+        <v>199</v>
+      </c>
+      <c r="C39" t="n">
+        <v>430082</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3864</v>
+      </c>
+      <c r="E39" t="n">
+        <v>644</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: crawl 08/07 21:48 VN (199 videos, +8); 37 dealers; today 11 videos
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,16 +458,16 @@
         <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>3074</v>
+        <v>2985</v>
       </c>
       <c r="D2" t="n">
         <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F2" t="n">
-        <v>3.74</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="3">
@@ -480,7 +480,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>2568</v>
+        <v>2551</v>
       </c>
       <c r="D3" t="n">
         <v>170</v>
@@ -489,7 +489,7 @@
         <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>7.63</v>
+        <v>7.68</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>384464</v>
+        <v>360342</v>
       </c>
       <c r="D4" t="n">
-        <v>2276</v>
+        <v>2154</v>
       </c>
       <c r="E4" t="n">
-        <v>405</v>
+        <v>369</v>
       </c>
       <c r="F4" t="n">
         <v>0.7</v>
@@ -524,7 +524,7 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>2011</v>
+        <v>1983</v>
       </c>
       <c r="D5" t="n">
         <v>48</v>
@@ -533,7 +533,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.39</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>1473</v>
+        <v>1440</v>
       </c>
       <c r="D6" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E6" t="n">
         <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>10.39</v>
+        <v>10.56</v>
       </c>
     </row>
     <row r="7">
@@ -568,7 +568,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>1485</v>
+        <v>1473</v>
       </c>
       <c r="D7" t="n">
         <v>28</v>
@@ -577,7 +577,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="8">
@@ -590,16 +590,16 @@
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>6936</v>
+        <v>6910</v>
       </c>
       <c r="D8" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E8" t="n">
         <v>5</v>
       </c>
       <c r="F8" t="n">
-        <v>1.96</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="9">
@@ -612,7 +612,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>3193</v>
+        <v>3168</v>
       </c>
       <c r="D9" t="n">
         <v>51</v>
@@ -621,7 +621,7 @@
         <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>1.94</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="10">
@@ -656,7 +656,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>1096</v>
+        <v>1091</v>
       </c>
       <c r="D11" t="n">
         <v>15</v>
@@ -665,7 +665,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>1.64</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="12">
@@ -678,7 +678,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>1161</v>
+        <v>1151</v>
       </c>
       <c r="D12" t="n">
         <v>17</v>
@@ -687,7 +687,7 @@
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>1.64</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="13">
@@ -700,16 +700,16 @@
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>1517</v>
+        <v>1491</v>
       </c>
       <c r="D13" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E13" t="n">
         <v>27</v>
       </c>
       <c r="F13" t="n">
-        <v>4.42</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="D14" t="n">
         <v>26</v>
@@ -731,7 +731,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>4.55</v>
+        <v>4.56</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>1258</v>
+        <v>1195</v>
       </c>
       <c r="D15" t="n">
         <v>18</v>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>1.43</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="16">
@@ -766,16 +766,16 @@
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>1102</v>
+        <v>1053</v>
       </c>
       <c r="D16" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="D17" t="n">
         <v>27</v>
@@ -797,7 +797,7 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>3.79</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="18">
@@ -810,7 +810,7 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D18" t="n">
         <v>11</v>
@@ -832,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="D19" t="n">
         <v>14</v>
@@ -841,7 +841,7 @@
         <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>3.35</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="20">
@@ -854,16 +854,16 @@
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>1195</v>
+        <v>1186</v>
       </c>
       <c r="D20" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E20" t="n">
         <v>13</v>
       </c>
       <c r="F20" t="n">
-        <v>7.62</v>
+        <v>7.59</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="D21" t="n">
         <v>12</v>
@@ -898,7 +898,7 @@
         <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="D22" t="n">
         <v>11</v>
@@ -907,7 +907,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.24</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D23" t="n">
         <v>8</v>
@@ -929,7 +929,7 @@
         <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>2.42</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="D24" t="n">
         <v>10</v>
@@ -951,7 +951,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="25">
@@ -986,7 +986,7 @@
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2552</v>
+        <v>2541</v>
       </c>
       <c r="D26" t="n">
         <v>33</v>
@@ -995,7 +995,7 @@
         <v>15</v>
       </c>
       <c r="F26" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2493</v>
+        <v>2336</v>
       </c>
       <c r="D27" t="n">
         <v>566</v>
@@ -1017,7 +1017,7 @@
         <v>18</v>
       </c>
       <c r="F27" t="n">
-        <v>23.43</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="D28" t="n">
         <v>18</v>
@@ -1039,7 +1039,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.58</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D29" t="n">
         <v>7</v>
@@ -1061,7 +1061,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1083,7 +1083,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1.55</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="31">
@@ -1096,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D31" t="n">
         <v>2</v>
@@ -1105,7 +1105,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>1.26</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="32">
@@ -1140,7 +1140,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>1220</v>
+        <v>1201</v>
       </c>
       <c r="D33" t="n">
         <v>12</v>
@@ -1149,7 +1149,7 @@
         <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="34">
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>319</v>
+        <v>225</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.31</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="36">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D36" t="n">
         <v>3</v>
@@ -1215,7 +1215,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>2.48</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="37">
@@ -1250,16 +1250,16 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>2.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1272,13 +1272,13 @@
         <v>199</v>
       </c>
       <c r="C39" t="n">
-        <v>430082</v>
+        <v>405188</v>
       </c>
       <c r="D39" t="n">
-        <v>3864</v>
+        <v>3735</v>
       </c>
       <c r="E39" t="n">
-        <v>644</v>
+        <v>607</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
feat: dealer celebration page (celebrate.html) + winners.json export
Open-gift fireworks page vinh danh winner đọc từ output/winners.json.
Honor roll trên dashboard thêm link 'Mở quà vinh danh' per winner.
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,63 +455,63 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3365</v>
+      </c>
+      <c r="D2" t="n">
+        <v>109</v>
+      </c>
+      <c r="E2" t="n">
         <v>19</v>
       </c>
-      <c r="C2" t="n">
-        <v>2985</v>
-      </c>
-      <c r="D2" t="n">
-        <v>96</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18</v>
-      </c>
       <c r="F2" t="n">
-        <v>3.82</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="n">
-        <v>2551</v>
+        <v>1897</v>
       </c>
       <c r="D3" t="n">
-        <v>170</v>
+        <v>86</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="F3" t="n">
-        <v>7.68</v>
+        <v>8.49</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>360342</v>
+        <v>2632</v>
       </c>
       <c r="D4" t="n">
-        <v>2154</v>
+        <v>171</v>
       </c>
       <c r="E4" t="n">
-        <v>369</v>
+        <v>26</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7</v>
+        <v>7.48</v>
       </c>
     </row>
     <row r="5">
@@ -521,107 +521,107 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="n">
-        <v>1983</v>
+        <v>2108</v>
       </c>
       <c r="D5" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.42</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>1440</v>
+        <v>424166</v>
       </c>
       <c r="D6" t="n">
-        <v>77</v>
+        <v>2521</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>464</v>
       </c>
       <c r="F6" t="n">
-        <v>10.56</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>1473</v>
+        <v>3362</v>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>1.97</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>6910</v>
+        <v>1634</v>
       </c>
       <c r="D8" t="n">
-        <v>130</v>
+        <v>29</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>1.95</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>3168</v>
+        <v>7067</v>
       </c>
       <c r="D9" t="n">
-        <v>51</v>
+        <v>138</v>
       </c>
       <c r="E9" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
-        <v>1.96</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
         <v>11</v>
       </c>
       <c r="C10" t="n">
-        <v>1217</v>
+        <v>1227</v>
       </c>
       <c r="D10" t="n">
         <v>9</v>
@@ -643,7 +643,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="11">
@@ -653,19 +653,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>1091</v>
+        <v>1138</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>1.65</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="12">
@@ -675,195 +675,195 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>1151</v>
+        <v>1183</v>
       </c>
       <c r="D12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>1.65</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>1491</v>
+        <v>759</v>
       </c>
       <c r="D13" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E13" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="F13" t="n">
-        <v>4.43</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>701</v>
+        <v>1546</v>
       </c>
       <c r="D14" t="n">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="F14" t="n">
-        <v>4.56</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1412</v>
+      </c>
+      <c r="D15" t="n">
+        <v>30</v>
+      </c>
+      <c r="E15" t="n">
         <v>4</v>
       </c>
-      <c r="C15" t="n">
-        <v>1195</v>
-      </c>
-      <c r="D15" t="n">
-        <v>18</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
       <c r="F15" t="n">
-        <v>1.51</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>1053</v>
+        <v>1380</v>
       </c>
       <c r="D16" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>2.37</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>737</v>
+        <v>1300</v>
       </c>
       <c r="D17" t="n">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>3.8</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>521</v>
+        <v>746</v>
       </c>
       <c r="D18" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2.11</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>471</v>
+        <v>526</v>
       </c>
       <c r="D19" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>3.4</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>1186</v>
+        <v>479</v>
       </c>
       <c r="D20" t="n">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="E20" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>7.59</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>822</v>
+        <v>1116</v>
       </c>
       <c r="D21" t="n">
         <v>12</v>
@@ -885,7 +885,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1.58</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="D22" t="n">
         <v>11</v>
@@ -907,7 +907,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.26</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="D23" t="n">
         <v>8</v>
@@ -929,7 +929,7 @@
         <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>2.43</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="24">
@@ -942,16 +942,16 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>2.19</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="25">
@@ -979,45 +979,45 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2541</v>
+        <v>2724</v>
       </c>
       <c r="D26" t="n">
-        <v>33</v>
+        <v>566</v>
       </c>
       <c r="E26" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F26" t="n">
-        <v>1.89</v>
+        <v>21.66</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2336</v>
+        <v>2568</v>
       </c>
       <c r="D27" t="n">
-        <v>566</v>
+        <v>33</v>
       </c>
       <c r="E27" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>25</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>692</v>
+        <v>720</v>
       </c>
       <c r="D28" t="n">
         <v>18</v>
@@ -1039,7 +1039,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="29">
@@ -1052,214 +1052,214 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>420</v>
+        <v>640</v>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>2.14</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ecomi.vn.roborock</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>252</v>
+        <v>343</v>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1.59</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>ecomi.vn.roborock</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>166</v>
+        <v>266</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>1.2</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>2592</v>
+        <v>175</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0.15</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>1201</v>
+        <v>2592</v>
       </c>
       <c r="D33" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>1.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>501</v>
+        <v>1279</v>
       </c>
       <c r="D34" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>roborock.smart.li</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>225</v>
+        <v>529</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>0.44</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>roborock.smart.li</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>119</v>
+        <v>343</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>2.52</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>bepphuthai</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0.85</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>anhlinhgroup_73</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="39">
@@ -1269,16 +1269,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="C39" t="n">
-        <v>405188</v>
+        <v>473009</v>
       </c>
       <c r="D39" t="n">
-        <v>3735</v>
+        <v>4182</v>
       </c>
       <c r="E39" t="n">
-        <v>607</v>
+        <v>715</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
data: crawl 10/07 00:41 VN (225 videos, +12); week-2 progress live
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3652</v>
+      </c>
+      <c r="D2" t="n">
+        <v>119</v>
+      </c>
+      <c r="E2" t="n">
         <v>21</v>
       </c>
-      <c r="C2" t="n">
-        <v>3365</v>
-      </c>
-      <c r="D2" t="n">
-        <v>109</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19</v>
-      </c>
       <c r="F2" t="n">
-        <v>3.8</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" t="n">
-        <v>1897</v>
+        <v>2129</v>
       </c>
       <c r="D3" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E3" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F3" t="n">
-        <v>8.49</v>
+        <v>7.89</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>2632</v>
+        <v>2697</v>
       </c>
       <c r="D4" t="n">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E4" t="n">
         <v>26</v>
       </c>
       <c r="F4" t="n">
-        <v>7.48</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="5">
@@ -521,19 +521,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>2108</v>
+        <v>2175</v>
       </c>
       <c r="D5" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.47</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="6">
@@ -546,82 +546,82 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>424166</v>
+        <v>456765</v>
       </c>
       <c r="D6" t="n">
-        <v>2521</v>
+        <v>2741</v>
       </c>
       <c r="E6" t="n">
-        <v>464</v>
+        <v>514</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>3362</v>
+        <v>7583</v>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>146</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
-        <v>1.84</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>1634</v>
+        <v>3483</v>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>1.84</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>7067</v>
+        <v>1663</v>
       </c>
       <c r="D9" t="n">
-        <v>138</v>
+        <v>30</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>2.05</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="10">
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C10" t="n">
-        <v>1227</v>
+        <v>1229</v>
       </c>
       <c r="D10" t="n">
         <v>9</v>
@@ -653,129 +653,129 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>1138</v>
+        <v>1290</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>1.93</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>1183</v>
+        <v>1719</v>
       </c>
       <c r="D12" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>1.69</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" t="n">
-        <v>759</v>
+        <v>1306</v>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>4.74</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>1546</v>
+        <v>2001</v>
       </c>
       <c r="D14" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="E14" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4.46</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>1412</v>
+        <v>824</v>
       </c>
       <c r="D15" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>2.41</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>1380</v>
+        <v>1584</v>
       </c>
       <c r="D16" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F16" t="n">
-        <v>1.81</v>
+        <v>4.36</v>
       </c>
     </row>
     <row r="17">
@@ -788,16 +788,16 @@
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>1300</v>
+        <v>1581</v>
       </c>
       <c r="D17" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E17" t="n">
         <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>7.46</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="18">
@@ -810,7 +810,7 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="D18" t="n">
         <v>28</v>
@@ -819,139 +819,139 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3.89</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>526</v>
+        <v>726</v>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.09</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>479</v>
+        <v>526</v>
       </c>
       <c r="D20" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>3.34</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>1116</v>
+        <v>482</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>1.16</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>535</v>
+        <v>1176</v>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.24</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>499</v>
+        <v>536</v>
       </c>
       <c r="D23" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2.4</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>466</v>
+        <v>500</v>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>2.36</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="25">
@@ -986,16 +986,16 @@
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2724</v>
+        <v>2997</v>
       </c>
       <c r="D26" t="n">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E26" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F26" t="n">
-        <v>21.66</v>
+        <v>19.92</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2568</v>
+        <v>2592</v>
       </c>
       <c r="D27" t="n">
         <v>33</v>
@@ -1017,7 +1017,7 @@
         <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>1.87</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="28">
@@ -1030,16 +1030,16 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="D28" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="29">
@@ -1052,16 +1052,16 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>640</v>
+        <v>703</v>
       </c>
       <c r="D29" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E29" t="n">
         <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>343</v>
+        <v>424</v>
       </c>
       <c r="D30" t="n">
         <v>3</v>
@@ -1083,7 +1083,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.87</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="31">
@@ -1096,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D31" t="n">
         <v>6</v>
@@ -1105,7 +1105,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="32">
@@ -1118,16 +1118,16 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>175</v>
+        <v>261</v>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.86</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="33">
@@ -1162,7 +1162,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1279</v>
+        <v>1353</v>
       </c>
       <c r="D34" t="n">
         <v>13</v>
@@ -1171,7 +1171,7 @@
         <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>1.25</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="35">
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>529</v>
+        <v>563</v>
       </c>
       <c r="D35" t="n">
         <v>4</v>
@@ -1193,7 +1193,7 @@
         <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>1.13</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="36">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D36" t="n">
         <v>1</v>
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D37" t="n">
         <v>3</v>
@@ -1237,7 +1237,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>2.42</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="38">
@@ -1269,16 +1269,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C39" t="n">
-        <v>473009</v>
+        <v>509493</v>
       </c>
       <c r="D39" t="n">
-        <v>4182</v>
+        <v>4465</v>
       </c>
       <c r="E39" t="n">
-        <v>715</v>
+        <v>776</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-10 13:07 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,63 +455,63 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>3652</v>
+        <v>4521</v>
       </c>
       <c r="D2" t="n">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="E2" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F2" t="n">
-        <v>3.83</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>2129</v>
+        <v>3477</v>
       </c>
       <c r="D3" t="n">
-        <v>92</v>
+        <v>211</v>
       </c>
       <c r="E3" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>7.89</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>2697</v>
+        <v>2249</v>
       </c>
       <c r="D4" t="n">
-        <v>175</v>
+        <v>94</v>
       </c>
       <c r="E4" t="n">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="F4" t="n">
-        <v>7.45</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="5">
@@ -521,151 +521,151 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>2175</v>
+        <v>2491</v>
       </c>
       <c r="D5" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>2.48</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>456765</v>
+        <v>3916</v>
       </c>
       <c r="D6" t="n">
-        <v>2741</v>
+        <v>59</v>
       </c>
       <c r="E6" t="n">
-        <v>514</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>0.71</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
-        <v>7583</v>
+        <v>2257</v>
       </c>
       <c r="D7" t="n">
-        <v>146</v>
+        <v>41</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>2.04</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>3483</v>
+        <v>516279</v>
       </c>
       <c r="D8" t="n">
-        <v>52</v>
+        <v>3142</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>597</v>
       </c>
       <c r="F8" t="n">
-        <v>1.81</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>1663</v>
+        <v>8109</v>
       </c>
       <c r="D9" t="n">
-        <v>30</v>
+        <v>148</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>1.86</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>12</v>
       </c>
       <c r="C10" t="n">
-        <v>1229</v>
+        <v>1897</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>0.73</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11" t="n">
-        <v>1290</v>
+        <v>1231</v>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>2.09</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="12">
@@ -675,19 +675,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>1719</v>
+        <v>2226</v>
       </c>
       <c r="D12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>2.39</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="13">
@@ -700,7 +700,7 @@
         <v>7</v>
       </c>
       <c r="C13" t="n">
-        <v>1306</v>
+        <v>1397</v>
       </c>
       <c r="D13" t="n">
         <v>18</v>
@@ -709,7 +709,7 @@
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>1.53</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="14">
@@ -722,16 +722,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>2001</v>
+        <v>2108</v>
       </c>
       <c r="D14" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1.5</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="D15" t="n">
         <v>33</v>
@@ -753,7 +753,7 @@
         <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>4.73</v>
+        <v>4.69</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>1584</v>
+        <v>1614</v>
       </c>
       <c r="D16" t="n">
         <v>42</v>
@@ -775,51 +775,51 @@
         <v>27</v>
       </c>
       <c r="F16" t="n">
-        <v>4.36</v>
+        <v>4.28</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" t="n">
-        <v>1581</v>
+        <v>1561</v>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>6.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>749</v>
+        <v>1616</v>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>3.87</v>
+        <v>6.19</v>
       </c>
     </row>
     <row r="19">
@@ -832,82 +832,82 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>726</v>
+        <v>833</v>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.2</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>526</v>
+        <v>756</v>
       </c>
       <c r="D20" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2.09</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>482</v>
+        <v>532</v>
       </c>
       <c r="D21" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>3.32</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>1176</v>
+        <v>486</v>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>1.11</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D23" t="n">
         <v>11</v>
@@ -929,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2.24</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="D24" t="n">
         <v>8</v>
@@ -951,7 +951,7 @@
         <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>2.4</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="25">
@@ -986,16 +986,16 @@
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>2997</v>
+        <v>3289</v>
       </c>
       <c r="D26" t="n">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="E26" t="n">
         <v>28</v>
       </c>
       <c r="F26" t="n">
-        <v>19.92</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2592</v>
+        <v>2607</v>
       </c>
       <c r="D27" t="n">
         <v>33</v>
@@ -1017,7 +1017,7 @@
         <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>731</v>
+        <v>752</v>
       </c>
       <c r="D28" t="n">
         <v>19</v>
@@ -1039,7 +1039,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.6</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="D29" t="n">
         <v>10</v>
@@ -1061,7 +1061,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.71</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="D30" t="n">
         <v>3</v>
@@ -1083,51 +1083,51 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ecomi.vn.roborock</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.25</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>ecomi.vn.roborock</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.68</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>2592</v>
+        <v>2593</v>
       </c>
       <c r="D33" t="n">
         <v>4</v>
@@ -1162,7 +1162,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1353</v>
+        <v>1403</v>
       </c>
       <c r="D34" t="n">
         <v>13</v>
@@ -1171,7 +1171,7 @@
         <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="35">
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>563</v>
+        <v>595</v>
       </c>
       <c r="D35" t="n">
         <v>4</v>
@@ -1193,7 +1193,7 @@
         <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>1.07</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="36">
@@ -1269,16 +1269,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="C39" t="n">
-        <v>509493</v>
+        <v>574995</v>
       </c>
       <c r="D39" t="n">
-        <v>4465</v>
+        <v>4974</v>
       </c>
       <c r="E39" t="n">
-        <v>776</v>
+        <v>871</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-11 11:50 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C2" t="n">
-        <v>4521</v>
+        <v>5032</v>
       </c>
       <c r="D2" t="n">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="E2" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>3.72</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>3477</v>
+        <v>3957</v>
       </c>
       <c r="D3" t="n">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="E3" t="n">
         <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>6.82</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="4">
@@ -499,63 +499,63 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>2249</v>
+        <v>2538</v>
       </c>
       <c r="D4" t="n">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E4" t="n">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="F4" t="n">
-        <v>7.69</v>
+        <v>8.470000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" t="n">
-        <v>2491</v>
+        <v>4398</v>
       </c>
       <c r="D5" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>2.45</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>3916</v>
+        <v>2569</v>
       </c>
       <c r="D6" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>1.79</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>15</v>
       </c>
       <c r="C7" t="n">
-        <v>2257</v>
+        <v>2565</v>
       </c>
       <c r="D7" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>1.86</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="8">
@@ -590,13 +590,13 @@
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>516279</v>
+        <v>526921</v>
       </c>
       <c r="D8" t="n">
-        <v>3142</v>
+        <v>3189</v>
       </c>
       <c r="E8" t="n">
-        <v>597</v>
+        <v>617</v>
       </c>
       <c r="F8" t="n">
         <v>0.72</v>
@@ -605,45 +605,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>8109</v>
+        <v>2534</v>
       </c>
       <c r="D9" t="n">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="E9" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>1.96</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B10" t="n">
+        <v>13</v>
+      </c>
+      <c r="C10" t="n">
+        <v>8280</v>
+      </c>
+      <c r="D10" t="n">
+        <v>159</v>
+      </c>
+      <c r="E10" t="n">
         <v>12</v>
       </c>
-      <c r="C10" t="n">
-        <v>1897</v>
-      </c>
-      <c r="D10" t="n">
-        <v>28</v>
-      </c>
-      <c r="E10" t="n">
-        <v>3</v>
-      </c>
       <c r="F10" t="n">
-        <v>1.63</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="11">
@@ -656,7 +656,7 @@
         <v>12</v>
       </c>
       <c r="C11" t="n">
-        <v>1231</v>
+        <v>1239</v>
       </c>
       <c r="D11" t="n">
         <v>9</v>
@@ -675,63 +675,63 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>2226</v>
+        <v>2799</v>
       </c>
       <c r="D12" t="n">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="E12" t="n">
         <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>2.29</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C13" t="n">
-        <v>1397</v>
+        <v>2435</v>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1.43</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>2108</v>
+        <v>1645</v>
       </c>
       <c r="D14" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>1.52</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="15">
@@ -741,63 +741,63 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>831</v>
+        <v>965</v>
       </c>
       <c r="D15" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E15" t="n">
         <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>4.69</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>1614</v>
+        <v>2255</v>
       </c>
       <c r="D16" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E16" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>4.28</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>5</v>
       </c>
       <c r="C17" t="n">
-        <v>1561</v>
+        <v>1664</v>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="F17" t="n">
-        <v>0.9</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1616</v>
+        <v>1656</v>
       </c>
       <c r="D18" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.19</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>833</v>
+        <v>847</v>
       </c>
       <c r="D19" t="n">
         <v>16</v>
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.04</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="D20" t="n">
         <v>28</v>
@@ -863,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.84</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="D21" t="n">
         <v>12</v>
@@ -885,7 +885,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.26</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -907,7 +907,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>3.29</v>
+        <v>3.28</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="D23" t="n">
         <v>11</v>
@@ -929,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2.22</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="D24" t="n">
         <v>8</v>
@@ -951,7 +951,7 @@
         <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>2.38</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="25">
@@ -986,16 +986,16 @@
         <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>3289</v>
+        <v>3553</v>
       </c>
       <c r="D26" t="n">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E26" t="n">
         <v>28</v>
       </c>
       <c r="F26" t="n">
-        <v>18.18</v>
+        <v>16.86</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2607</v>
+        <v>2625</v>
       </c>
       <c r="D27" t="n">
         <v>33</v>
@@ -1017,7 +1017,7 @@
         <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>1.84</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>752</v>
+        <v>767</v>
       </c>
       <c r="D28" t="n">
         <v>19</v>
@@ -1039,7 +1039,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.53</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="D29" t="n">
         <v>10</v>
@@ -1061,7 +1061,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.68</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="D30" t="n">
         <v>3</v>
@@ -1096,16 +1096,16 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="D31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.55</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="32">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="D32" t="n">
         <v>6</v>
@@ -1127,160 +1127,204 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.22</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>2593</v>
+        <v>96</v>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0.15</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1403</v>
+        <v>2593</v>
       </c>
       <c r="D34" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>1.14</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>595</v>
+        <v>1442</v>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>1.01</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>roborock.smart.li</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>346</v>
+        <v>657</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>0.29</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>roborock.smart.li</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>125</v>
+        <v>346</v>
       </c>
       <c r="D37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>2.4</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>bepphuthai</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.83</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>anhlinhgroup_73</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>120</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>homebotvietnam</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>86</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>254</v>
-      </c>
-      <c r="C39" t="n">
-        <v>574995</v>
-      </c>
-      <c r="D39" t="n">
-        <v>4974</v>
-      </c>
-      <c r="E39" t="n">
-        <v>871</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="B41" t="n">
+        <v>277</v>
+      </c>
+      <c r="C41" t="n">
+        <v>591316</v>
+      </c>
+      <c r="D41" t="n">
+        <v>5159</v>
+      </c>
+      <c r="E41" t="n">
+        <v>917</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-12 11:56 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C2" t="n">
-        <v>5032</v>
+        <v>5635</v>
       </c>
       <c r="D2" t="n">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="E2" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="F2" t="n">
-        <v>3.76</v>
+        <v>4.44</v>
       </c>
     </row>
     <row r="3">
@@ -480,38 +480,38 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>3957</v>
+        <v>4107</v>
       </c>
       <c r="D3" t="n">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="E3" t="n">
         <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>6.47</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4" t="n">
-        <v>2538</v>
+        <v>3584</v>
       </c>
       <c r="D4" t="n">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="E4" t="n">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>8.470000000000001</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="5">
@@ -521,107 +521,107 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C5" t="n">
-        <v>4398</v>
+        <v>5490</v>
       </c>
       <c r="D5" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5" t="n">
         <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>1.86</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" t="n">
-        <v>2569</v>
+        <v>4344</v>
       </c>
       <c r="D6" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>2.69</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>2565</v>
+        <v>2650</v>
       </c>
       <c r="D7" t="n">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="F7" t="n">
-        <v>1.87</v>
+        <v>8.23</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" t="n">
-        <v>526921</v>
+        <v>3323</v>
       </c>
       <c r="D8" t="n">
-        <v>3189</v>
+        <v>40</v>
       </c>
       <c r="E8" t="n">
-        <v>617</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>0.72</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>2534</v>
+        <v>625059</v>
       </c>
       <c r="D9" t="n">
-        <v>35</v>
+        <v>3864</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>717</v>
       </c>
       <c r="F9" t="n">
-        <v>1.5</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="10">
@@ -634,60 +634,60 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>8280</v>
+        <v>8653</v>
       </c>
       <c r="D10" t="n">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E10" t="n">
         <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>2.07</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>12</v>
       </c>
       <c r="C11" t="n">
-        <v>1239</v>
+        <v>3220</v>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
-        <v>0.73</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>2799</v>
+        <v>1243</v>
       </c>
       <c r="D12" t="n">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>2.22</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="13">
@@ -697,19 +697,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>2435</v>
+        <v>3072</v>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
-        <v>1.56</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="14">
@@ -719,19 +719,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C14" t="n">
-        <v>1645</v>
+        <v>1948</v>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>1.28</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>965</v>
+        <v>1173</v>
       </c>
       <c r="D15" t="n">
         <v>36</v>
@@ -753,7 +753,7 @@
         <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>4.35</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>2255</v>
+        <v>2282</v>
       </c>
       <c r="D16" t="n">
         <v>19</v>
@@ -775,7 +775,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="17">
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>1664</v>
+        <v>1845</v>
       </c>
       <c r="D17" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E17" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F17" t="n">
-        <v>4.21</v>
+        <v>4.07</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1656</v>
+        <v>1678</v>
       </c>
       <c r="D18" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.22</v>
+        <v>6.32</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>847</v>
+        <v>855</v>
       </c>
       <c r="D19" t="n">
         <v>16</v>
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.01</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="D20" t="n">
         <v>28</v>
@@ -863,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.8</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="D21" t="n">
         <v>12</v>
@@ -885,7 +885,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.23</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -907,7 +907,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>3.28</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="D23" t="n">
         <v>11</v>
@@ -929,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="D24" t="n">
         <v>8</v>
@@ -951,205 +951,205 @@
         <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>43</v>
+        <v>396</v>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>20.93</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>3553</v>
+        <v>43</v>
       </c>
       <c r="D26" t="n">
-        <v>571</v>
+        <v>9</v>
       </c>
       <c r="E26" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>16.86</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>2625</v>
+        <v>4127</v>
       </c>
       <c r="D27" t="n">
-        <v>33</v>
+        <v>576</v>
       </c>
       <c r="E27" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>1.83</v>
+        <v>14.68</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>767</v>
+        <v>2652</v>
       </c>
       <c r="D28" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F28" t="n">
-        <v>2.48</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>720</v>
+        <v>784</v>
       </c>
       <c r="D29" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>1.67</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>436</v>
+        <v>726</v>
       </c>
       <c r="D30" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>288</v>
+        <v>438</v>
       </c>
       <c r="D31" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.78</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ecomi.vn.roborock</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.18</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>ecomi.vn.roborock</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>96</v>
+        <v>277</v>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.08</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="34">
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>1442</v>
+        <v>1493</v>
       </c>
       <c r="D35" t="n">
         <v>13</v>
@@ -1193,7 +1193,7 @@
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>1.11</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="36">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>657</v>
+        <v>731</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
@@ -1215,7 +1215,7 @@
         <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>0.91</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="37">
@@ -1243,14 +1243,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>125</v>
+        <v>185</v>
       </c>
       <c r="D38" t="n">
         <v>3</v>
@@ -1259,51 +1259,51 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>2.4</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>bepphuthai</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0.83</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>anhlinhgroup_73</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>2.33</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="41">
@@ -1313,16 +1313,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>277</v>
+        <v>304</v>
       </c>
       <c r="C41" t="n">
-        <v>591316</v>
+        <v>698354</v>
       </c>
       <c r="D41" t="n">
-        <v>5159</v>
+        <v>5999</v>
       </c>
       <c r="E41" t="n">
-        <v>917</v>
+        <v>1048</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-13 13:15 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" t="n">
-        <v>5635</v>
+        <v>6122</v>
       </c>
       <c r="D2" t="n">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="E2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F2" t="n">
-        <v>4.44</v>
+        <v>4.38</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>4107</v>
+        <v>4189</v>
       </c>
       <c r="D3" t="n">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="E3" t="n">
         <v>26</v>
       </c>
       <c r="F3" t="n">
-        <v>6.53</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>23</v>
       </c>
       <c r="C4" t="n">
-        <v>3584</v>
+        <v>3745</v>
       </c>
       <c r="D4" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>2.79</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>21</v>
       </c>
       <c r="C5" t="n">
-        <v>5490</v>
+        <v>5785</v>
       </c>
       <c r="D5" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E5" t="n">
         <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>1.53</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>21</v>
       </c>
       <c r="C6" t="n">
-        <v>4344</v>
+        <v>4734</v>
       </c>
       <c r="D6" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
-        <v>1.57</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>2650</v>
+        <v>2699</v>
       </c>
       <c r="D7" t="n">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="E7" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F7" t="n">
-        <v>8.23</v>
+        <v>8.859999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -590,16 +590,16 @@
         <v>15</v>
       </c>
       <c r="C8" t="n">
-        <v>3323</v>
+        <v>3607</v>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="9">
@@ -612,13 +612,13 @@
         <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>625059</v>
+        <v>638286</v>
       </c>
       <c r="D9" t="n">
-        <v>3864</v>
+        <v>3953</v>
       </c>
       <c r="E9" t="n">
-        <v>717</v>
+        <v>735</v>
       </c>
       <c r="F9" t="n">
         <v>0.73</v>
@@ -634,16 +634,16 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>8653</v>
+        <v>8751</v>
       </c>
       <c r="D10" t="n">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E10" t="n">
         <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="11">
@@ -653,85 +653,85 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" t="n">
-        <v>3220</v>
+        <v>3352</v>
       </c>
       <c r="D11" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E11" t="n">
         <v>8</v>
       </c>
       <c r="F11" t="n">
-        <v>2.27</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>1243</v>
+        <v>4016</v>
       </c>
       <c r="D12" t="n">
-        <v>9</v>
+        <v>112</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F12" t="n">
-        <v>0.72</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>3072</v>
+        <v>2148</v>
       </c>
       <c r="D13" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>2.02</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1948</v>
+        <v>1260</v>
       </c>
       <c r="D14" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>1.33</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>1173</v>
+        <v>1183</v>
       </c>
       <c r="D15" t="n">
         <v>36</v>
@@ -753,7 +753,7 @@
         <v>6</v>
       </c>
       <c r="F15" t="n">
-        <v>3.58</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>2282</v>
+        <v>2299</v>
       </c>
       <c r="D16" t="n">
         <v>19</v>
@@ -775,7 +775,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="17">
@@ -788,16 +788,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>1845</v>
+        <v>1879</v>
       </c>
       <c r="D17" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E17" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>4.07</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1678</v>
+        <v>1717</v>
       </c>
       <c r="D18" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.32</v>
+        <v>6.29</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>855</v>
+        <v>867</v>
       </c>
       <c r="D19" t="n">
         <v>16</v>
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="20">
@@ -869,111 +869,111 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>542</v>
+        <v>661</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.21</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>494</v>
+        <v>546</v>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>3.24</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>549</v>
+        <v>494</v>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>2.19</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>515</v>
+        <v>563</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>2.33</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>396</v>
+        <v>519</v>
       </c>
       <c r="D25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" t="n">
         <v>4</v>
       </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
       <c r="F25" t="n">
-        <v>1.01</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="26">
@@ -1008,16 +1008,16 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>4127</v>
+        <v>4806</v>
       </c>
       <c r="D27" t="n">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="E27" t="n">
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>14.68</v>
+        <v>12.73</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>2652</v>
+        <v>2675</v>
       </c>
       <c r="D28" t="n">
         <v>33</v>
@@ -1039,7 +1039,7 @@
         <v>15</v>
       </c>
       <c r="F28" t="n">
-        <v>1.81</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>784</v>
+        <v>798</v>
       </c>
       <c r="D29" t="n">
         <v>20</v>
@@ -1061,7 +1061,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.55</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="D30" t="n">
         <v>10</v>
@@ -1096,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D31" t="n">
         <v>3</v>
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D32" t="n">
         <v>8</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.78</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="33">
@@ -1162,7 +1162,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>2593</v>
+        <v>2597</v>
       </c>
       <c r="D34" t="n">
         <v>4</v>
@@ -1184,16 +1184,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>1493</v>
+        <v>1542</v>
       </c>
       <c r="D35" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>1.07</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="36">
@@ -1206,16 +1206,16 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>731</v>
+        <v>810</v>
       </c>
       <c r="D36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" t="n">
         <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="37">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D37" t="n">
         <v>1</v>
@@ -1250,7 +1250,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>185</v>
+        <v>206</v>
       </c>
       <c r="D38" t="n">
         <v>3</v>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>1.62</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="39">
@@ -1272,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D39" t="n">
         <v>3</v>
@@ -1281,7 +1281,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>2.4</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="40">
@@ -1313,16 +1313,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C41" t="n">
-        <v>698354</v>
+        <v>715998</v>
       </c>
       <c r="D41" t="n">
-        <v>5999</v>
+        <v>6228</v>
       </c>
       <c r="E41" t="n">
-        <v>1048</v>
+        <v>1100</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-14 12:13 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,107 +455,107 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C2" t="n">
-        <v>6122</v>
+        <v>6729</v>
       </c>
       <c r="D2" t="n">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="E2" t="n">
         <v>45</v>
       </c>
       <c r="F2" t="n">
-        <v>4.38</v>
+        <v>4.12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C3" t="n">
-        <v>4189</v>
+        <v>5234</v>
       </c>
       <c r="D3" t="n">
-        <v>246</v>
+        <v>132</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>6.49</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" t="n">
-        <v>3745</v>
+        <v>4250</v>
       </c>
       <c r="D4" t="n">
-        <v>105</v>
+        <v>249</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="F4" t="n">
-        <v>2.86</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="n">
-        <v>5785</v>
+        <v>4990</v>
       </c>
       <c r="D5" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>1.47</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>21</v>
       </c>
       <c r="C6" t="n">
-        <v>4734</v>
+        <v>5896</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
-        <v>1.71</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="7">
@@ -568,104 +568,104 @@
         <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>2699</v>
+        <v>2742</v>
       </c>
       <c r="D7" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E7" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F7" t="n">
-        <v>8.859999999999999</v>
+        <v>8.789999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>15</v>
       </c>
       <c r="C8" t="n">
-        <v>3607</v>
+        <v>3887</v>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>1.3</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
-        <v>638286</v>
+        <v>3675</v>
       </c>
       <c r="D9" t="n">
-        <v>3953</v>
+        <v>48</v>
       </c>
       <c r="E9" t="n">
-        <v>735</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>0.73</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C10" t="n">
-        <v>8751</v>
+        <v>648357</v>
       </c>
       <c r="D10" t="n">
-        <v>165</v>
+        <v>3993</v>
       </c>
       <c r="E10" t="n">
-        <v>12</v>
+        <v>746</v>
       </c>
       <c r="F10" t="n">
-        <v>2.02</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>13</v>
       </c>
       <c r="C11" t="n">
-        <v>3352</v>
+        <v>8837</v>
       </c>
       <c r="D11" t="n">
-        <v>67</v>
+        <v>166</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>2.24</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="12">
@@ -678,16 +678,16 @@
         <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>4016</v>
+        <v>4490</v>
       </c>
       <c r="D12" t="n">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E12" t="n">
         <v>18</v>
       </c>
       <c r="F12" t="n">
-        <v>3.24</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="13">
@@ -700,16 +700,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>2148</v>
+        <v>2372</v>
       </c>
       <c r="D13" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>1.3</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="14">
@@ -722,16 +722,16 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.71</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="15">
@@ -744,16 +744,16 @@
         <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>1183</v>
+        <v>1189</v>
       </c>
       <c r="D15" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
-        <v>3.55</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>2299</v>
+        <v>2311</v>
       </c>
       <c r="D16" t="n">
         <v>19</v>
@@ -788,16 +788,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>1879</v>
+        <v>1912</v>
       </c>
       <c r="D17" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E17" t="n">
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>4.2</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1717</v>
+        <v>1741</v>
       </c>
       <c r="D18" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.29</v>
+        <v>6.32</v>
       </c>
     </row>
     <row r="19">
@@ -832,16 +832,16 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>867</v>
+        <v>879</v>
       </c>
       <c r="D19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1.96</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>765</v>
+        <v>773</v>
       </c>
       <c r="D20" t="n">
         <v>28</v>
@@ -863,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.79</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>661</v>
+        <v>717</v>
       </c>
       <c r="D21" t="n">
         <v>14</v>
@@ -885,7 +885,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.27</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="22">
@@ -898,16 +898,16 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2.2</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -929,7 +929,7 @@
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>3.24</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="D24" t="n">
         <v>10</v>
@@ -951,7 +951,7 @@
         <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>3.02</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="25">
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D25" t="n">
         <v>8</v>
@@ -973,7 +973,7 @@
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>2.31</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="26">
@@ -1008,16 +1008,16 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>4806</v>
+        <v>5112</v>
       </c>
       <c r="D27" t="n">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E27" t="n">
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>12.73</v>
+        <v>12.01</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>2675</v>
+        <v>2754</v>
       </c>
       <c r="D28" t="n">
         <v>33</v>
@@ -1039,7 +1039,7 @@
         <v>15</v>
       </c>
       <c r="F28" t="n">
-        <v>1.79</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="29">
@@ -1052,16 +1052,16 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>798</v>
+        <v>812</v>
       </c>
       <c r="D29" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.51</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="D30" t="n">
         <v>10</v>
@@ -1083,7 +1083,7 @@
         <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>1.65</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="31">
@@ -1096,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D31" t="n">
         <v>3</v>
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D32" t="n">
         <v>8</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.77</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D33" t="n">
         <v>6</v>
@@ -1149,51 +1149,51 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.17</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>2597</v>
+        <v>3286</v>
       </c>
       <c r="D34" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>0.15</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>1542</v>
+        <v>2598</v>
       </c>
       <c r="D35" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>1.17</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="36">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>810</v>
+        <v>875</v>
       </c>
       <c r="D36" t="n">
         <v>5</v>
@@ -1215,7 +1215,7 @@
         <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>0.86</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="37">
@@ -1250,7 +1250,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="D38" t="n">
         <v>3</v>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>1.46</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="39">
@@ -1272,16 +1272,16 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>2.33</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="40">
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
@@ -1303,7 +1303,7 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="41">
@@ -1313,16 +1313,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="C41" t="n">
-        <v>715998</v>
+        <v>732436</v>
       </c>
       <c r="D41" t="n">
-        <v>6228</v>
+        <v>6368</v>
       </c>
       <c r="E41" t="n">
-        <v>1100</v>
+        <v>1120</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-15 12:18 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C2" t="n">
-        <v>6729</v>
+        <v>7937</v>
       </c>
       <c r="D2" t="n">
-        <v>232</v>
+        <v>263</v>
       </c>
       <c r="E2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F2" t="n">
-        <v>4.12</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>30</v>
       </c>
       <c r="C3" t="n">
-        <v>5234</v>
+        <v>5687</v>
       </c>
       <c r="D3" t="n">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>2.64</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="4">
@@ -502,60 +502,60 @@
         <v>24</v>
       </c>
       <c r="C4" t="n">
-        <v>4250</v>
+        <v>4287</v>
       </c>
       <c r="D4" t="n">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E4" t="n">
         <v>26</v>
       </c>
       <c r="F4" t="n">
-        <v>6.47</v>
+        <v>6.46</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" t="n">
-        <v>4990</v>
+        <v>6214</v>
       </c>
       <c r="D5" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F5" t="n">
-        <v>1.72</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" t="n">
-        <v>5896</v>
+        <v>5090</v>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>1.44</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" t="n">
-        <v>2742</v>
+        <v>2886</v>
       </c>
       <c r="D7" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E7" t="n">
         <v>107</v>
       </c>
       <c r="F7" t="n">
-        <v>8.789999999999999</v>
+        <v>8.42</v>
       </c>
     </row>
     <row r="8">
@@ -587,19 +587,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C8" t="n">
-        <v>3887</v>
+        <v>4972</v>
       </c>
       <c r="D8" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>2.14</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="9">
@@ -609,10 +609,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9" t="n">
-        <v>3675</v>
+        <v>3961</v>
       </c>
       <c r="D9" t="n">
         <v>48</v>
@@ -621,7 +621,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>1.39</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="10">
@@ -634,13 +634,13 @@
         <v>14</v>
       </c>
       <c r="C10" t="n">
-        <v>648357</v>
+        <v>654957</v>
       </c>
       <c r="D10" t="n">
-        <v>3993</v>
+        <v>4034</v>
       </c>
       <c r="E10" t="n">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="F10" t="n">
         <v>0.73</v>
@@ -649,45 +649,45 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>8837</v>
+        <v>5074</v>
       </c>
       <c r="D11" t="n">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F11" t="n">
-        <v>2.01</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B12" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" t="n">
+        <v>8903</v>
+      </c>
+      <c r="D12" t="n">
+        <v>169</v>
+      </c>
+      <c r="E12" t="n">
         <v>12</v>
       </c>
-      <c r="C12" t="n">
-        <v>4490</v>
-      </c>
-      <c r="D12" t="n">
-        <v>126</v>
-      </c>
-      <c r="E12" t="n">
-        <v>18</v>
-      </c>
       <c r="F12" t="n">
-        <v>3.21</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="13">
@@ -697,19 +697,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>2372</v>
+        <v>2825</v>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>1.35</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="D14" t="n">
         <v>10</v>
@@ -737,45 +737,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>1189</v>
+        <v>2697</v>
       </c>
       <c r="D15" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>3.7</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>2311</v>
+        <v>1192</v>
       </c>
       <c r="D16" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
-        <v>0.87</v>
+        <v>3.78</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>1912</v>
+        <v>1958</v>
       </c>
       <c r="D17" t="n">
         <v>50</v>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>4.18</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1741</v>
+        <v>1782</v>
       </c>
       <c r="D18" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.32</v>
+        <v>6.29</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>879</v>
+        <v>892</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.05</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="D20" t="n">
         <v>28</v>
@@ -863,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.75</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>717</v>
+        <v>727</v>
       </c>
       <c r="D21" t="n">
         <v>14</v>
@@ -885,7 +885,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.09</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D22" t="n">
         <v>13</v>
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -929,7 +929,7 @@
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>3.23</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="D24" t="n">
         <v>10</v>
@@ -951,7 +951,7 @@
         <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>2.96</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="25">
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="D25" t="n">
         <v>8</v>
@@ -973,7 +973,7 @@
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>2.3</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="26">
@@ -1008,16 +1008,16 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>5112</v>
+        <v>5408</v>
       </c>
       <c r="D27" t="n">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E27" t="n">
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>12.01</v>
+        <v>11.43</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>2754</v>
+        <v>2848</v>
       </c>
       <c r="D28" t="n">
         <v>33</v>
@@ -1039,7 +1039,7 @@
         <v>15</v>
       </c>
       <c r="F28" t="n">
-        <v>1.74</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>812</v>
+        <v>824</v>
       </c>
       <c r="D29" t="n">
         <v>21</v>
@@ -1061,7 +1061,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.59</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="30">
@@ -1074,7 +1074,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="D30" t="n">
         <v>10</v>
@@ -1089,14 +1089,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>440</v>
+        <v>615</v>
       </c>
       <c r="D31" t="n">
         <v>3</v>
@@ -1105,161 +1105,161 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0.68</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>294</v>
+        <v>441</v>
       </c>
       <c r="D32" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.72</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ecomi.vn.roborock</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.16</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>ecomi.vn.roborock</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>3286</v>
+        <v>278</v>
       </c>
       <c r="D34" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>1.03</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>2598</v>
+        <v>15100</v>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>0.15</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>875</v>
+        <v>2599</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>roborock.smart.li</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>348</v>
+        <v>981</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>0.29</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.smart.li</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>224</v>
+        <v>348</v>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>1.34</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="39">
@@ -1272,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D39" t="n">
         <v>4</v>
@@ -1281,7 +1281,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>3.05</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="40">
@@ -1313,16 +1313,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>321</v>
+        <v>341</v>
       </c>
       <c r="C41" t="n">
-        <v>732436</v>
+        <v>757002</v>
       </c>
       <c r="D41" t="n">
-        <v>6368</v>
+        <v>6561</v>
       </c>
       <c r="E41" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-16 12:23 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C2" t="n">
-        <v>7937</v>
+        <v>8974</v>
       </c>
       <c r="D2" t="n">
-        <v>263</v>
+        <v>286</v>
       </c>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>3.94</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="3">
@@ -477,85 +477,85 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C3" t="n">
-        <v>5687</v>
+        <v>6312</v>
       </c>
       <c r="D3" t="n">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>2.73</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>24</v>
       </c>
       <c r="C4" t="n">
-        <v>4287</v>
+        <v>5390</v>
       </c>
       <c r="D4" t="n">
-        <v>251</v>
+        <v>85</v>
       </c>
       <c r="E4" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>6.46</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" t="n">
-        <v>6214</v>
+        <v>4427</v>
       </c>
       <c r="D5" t="n">
-        <v>74</v>
+        <v>262</v>
       </c>
       <c r="E5" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>1.42</v>
+        <v>6.51</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="n">
-        <v>5090</v>
+        <v>6295</v>
       </c>
       <c r="D6" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>1.75</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="7">
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" t="n">
-        <v>2886</v>
+        <v>2971</v>
       </c>
       <c r="D7" t="n">
         <v>136</v>
@@ -577,7 +577,7 @@
         <v>107</v>
       </c>
       <c r="F7" t="n">
-        <v>8.42</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="8">
@@ -587,19 +587,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" t="n">
-        <v>4972</v>
+        <v>5370</v>
       </c>
       <c r="D8" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E8" t="n">
         <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>2.01</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="9">
@@ -609,107 +609,107 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>3961</v>
+        <v>4639</v>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>1.29</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" t="n">
-        <v>654957</v>
+        <v>3250</v>
       </c>
       <c r="D10" t="n">
-        <v>4034</v>
+        <v>38</v>
       </c>
       <c r="E10" t="n">
-        <v>750</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
-        <v>0.73</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>5074</v>
+        <v>659350</v>
       </c>
       <c r="D11" t="n">
-        <v>158</v>
+        <v>4054</v>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>750</v>
       </c>
       <c r="F11" t="n">
-        <v>3.49</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>8903</v>
+        <v>5185</v>
       </c>
       <c r="D12" t="n">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>2.03</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>2825</v>
+        <v>8938</v>
       </c>
       <c r="D13" t="n">
-        <v>35</v>
+        <v>171</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>1.31</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="D14" t="n">
         <v>10</v>
@@ -744,16 +744,16 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>2697</v>
+        <v>3001</v>
       </c>
       <c r="D15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>1192</v>
+        <v>1196</v>
       </c>
       <c r="D16" t="n">
         <v>38</v>
@@ -775,7 +775,7 @@
         <v>7</v>
       </c>
       <c r="F16" t="n">
-        <v>3.78</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>1958</v>
+        <v>2004</v>
       </c>
       <c r="D17" t="n">
         <v>50</v>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>4.09</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1782</v>
+        <v>1808</v>
       </c>
       <c r="D18" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.29</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="19">
@@ -832,16 +832,16 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>892</v>
+        <v>902</v>
       </c>
       <c r="D19" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.02</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="D20" t="n">
         <v>28</v>
@@ -863,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.74</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="21">
@@ -876,16 +876,16 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>727</v>
+        <v>757</v>
       </c>
       <c r="D21" t="n">
         <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.06</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="D22" t="n">
         <v>13</v>
@@ -907,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -929,7 +929,7 @@
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>3.22</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="D24" t="n">
         <v>10</v>
@@ -951,174 +951,174 @@
         <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>2.95</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>525</v>
+        <v>570</v>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.29</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>43</v>
+        <v>529</v>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>20.93</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5408</v>
+        <v>43</v>
       </c>
       <c r="D27" t="n">
-        <v>588</v>
+        <v>9</v>
       </c>
       <c r="E27" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>11.43</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>2</v>
       </c>
       <c r="C28" t="n">
-        <v>2848</v>
+        <v>5633</v>
       </c>
       <c r="D28" t="n">
-        <v>33</v>
+        <v>590</v>
       </c>
       <c r="E28" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F28" t="n">
-        <v>1.69</v>
+        <v>11.01</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>824</v>
+        <v>2851</v>
       </c>
       <c r="D29" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F29" t="n">
-        <v>2.55</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>737</v>
+        <v>825</v>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1.63</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>615</v>
+        <v>749</v>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>0.49</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>441</v>
+        <v>635</v>
       </c>
       <c r="D32" t="n">
         <v>3</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0.68</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="33">
@@ -1140,16 +1140,16 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.72</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="34">
@@ -1162,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D34" t="n">
         <v>6</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2.16</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="35">
@@ -1184,10 +1184,10 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>15100</v>
+        <v>24900</v>
       </c>
       <c r="D35" t="n">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>2599</v>
+        <v>2600</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>981</v>
+        <v>1096</v>
       </c>
       <c r="D37" t="n">
         <v>5</v>
@@ -1237,7 +1237,7 @@
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>0.71</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="38">
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
@@ -1303,7 +1303,7 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="41">
@@ -1313,16 +1313,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="C41" t="n">
-        <v>757002</v>
+        <v>776066</v>
       </c>
       <c r="D41" t="n">
-        <v>6561</v>
+        <v>6710</v>
       </c>
       <c r="E41" t="n">
-        <v>1140</v>
+        <v>1149</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-17 12:12 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
-        <v>8974</v>
+        <v>9965</v>
       </c>
       <c r="D2" t="n">
-        <v>286</v>
+        <v>304</v>
       </c>
       <c r="E2" t="n">
         <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>3.77</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="3">
@@ -477,151 +477,151 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C3" t="n">
-        <v>6312</v>
+        <v>6532</v>
       </c>
       <c r="D3" t="n">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>2.69</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C4" t="n">
-        <v>5390</v>
+        <v>5467</v>
       </c>
       <c r="D4" t="n">
-        <v>85</v>
+        <v>278</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F4" t="n">
-        <v>1.78</v>
+        <v>5.56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C5" t="n">
-        <v>4427</v>
+        <v>7362</v>
       </c>
       <c r="D5" t="n">
-        <v>262</v>
+        <v>84</v>
       </c>
       <c r="E5" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F5" t="n">
-        <v>6.51</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" t="n">
-        <v>6295</v>
+        <v>5533</v>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>1.43</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>22</v>
       </c>
       <c r="C7" t="n">
-        <v>2971</v>
+        <v>6253</v>
       </c>
       <c r="D7" t="n">
-        <v>136</v>
+        <v>57</v>
       </c>
       <c r="E7" t="n">
-        <v>107</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>8.18</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
-        <v>5370</v>
+        <v>3077</v>
       </c>
       <c r="D8" t="n">
-        <v>90</v>
+        <v>138</v>
       </c>
       <c r="E8" t="n">
-        <v>17</v>
+        <v>108</v>
       </c>
       <c r="F8" t="n">
-        <v>1.99</v>
+        <v>7.99</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9" t="n">
-        <v>4639</v>
+        <v>5801</v>
       </c>
       <c r="D9" t="n">
-        <v>52</v>
+        <v>103</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>1.19</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" t="n">
-        <v>3250</v>
+        <v>3859</v>
       </c>
       <c r="D10" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E10" t="n">
         <v>6</v>
       </c>
       <c r="F10" t="n">
-        <v>1.35</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="11">
@@ -656,13 +656,13 @@
         <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>659350</v>
+        <v>662547</v>
       </c>
       <c r="D11" t="n">
-        <v>4054</v>
+        <v>4061</v>
       </c>
       <c r="E11" t="n">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="F11" t="n">
         <v>0.73</v>
@@ -678,7 +678,7 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>5185</v>
+        <v>5251</v>
       </c>
       <c r="D12" t="n">
         <v>159</v>
@@ -687,7 +687,7 @@
         <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>3.43</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="13">
@@ -700,10 +700,10 @@
         <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>8938</v>
+        <v>8986</v>
       </c>
       <c r="D13" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -722,7 +722,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1263</v>
+        <v>1269</v>
       </c>
       <c r="D14" t="n">
         <v>10</v>
@@ -741,19 +741,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>3001</v>
+        <v>3745</v>
       </c>
       <c r="D15" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>1.07</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="16">
@@ -788,16 +788,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2004</v>
+        <v>2050</v>
       </c>
       <c r="D17" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E17" t="n">
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.99</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1808</v>
+        <v>1832</v>
       </c>
       <c r="D18" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E18" t="n">
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>6.25</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>902</v>
+        <v>911</v>
       </c>
       <c r="D19" t="n">
         <v>19</v>
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2.22</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="20">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>757</v>
+        <v>772</v>
       </c>
       <c r="D21" t="n">
         <v>14</v>
@@ -885,7 +885,7 @@
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.11</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D22" t="n">
         <v>13</v>
@@ -907,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -935,23 +935,23 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>583</v>
+        <v>673</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>2.92</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="25">
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>570</v>
+        <v>627</v>
       </c>
       <c r="D25" t="n">
         <v>7</v>
@@ -973,161 +973,161 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>1.23</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>529</v>
+        <v>583</v>
       </c>
       <c r="D26" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
-        <v>2.27</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>43</v>
+        <v>531</v>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>20.93</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>5633</v>
+        <v>43</v>
       </c>
       <c r="D28" t="n">
-        <v>590</v>
+        <v>9</v>
       </c>
       <c r="E28" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>11.01</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>2851</v>
+        <v>5806</v>
       </c>
       <c r="D29" t="n">
-        <v>33</v>
+        <v>592</v>
       </c>
       <c r="E29" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F29" t="n">
-        <v>1.68</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>825</v>
+        <v>2852</v>
       </c>
       <c r="D30" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F30" t="n">
-        <v>2.55</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>749</v>
+        <v>831</v>
       </c>
       <c r="D31" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>1.6</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>635</v>
+        <v>751</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>0.47</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="D33" t="n">
         <v>9</v>
@@ -1149,7 +1149,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>3.01</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="34">
@@ -1162,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D34" t="n">
         <v>6</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="35">
@@ -1184,16 +1184,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>24900</v>
+        <v>35800</v>
       </c>
       <c r="D35" t="n">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="36">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
@@ -1228,16 +1228,16 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1096</v>
+        <v>1194</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" t="n">
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="38">
@@ -1272,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D39" t="n">
         <v>4</v>
@@ -1281,7 +1281,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>3.03</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="40">
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
@@ -1303,7 +1303,7 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="41">
@@ -1313,16 +1313,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>357</v>
+        <v>389</v>
       </c>
       <c r="C41" t="n">
-        <v>776066</v>
+        <v>797732</v>
       </c>
       <c r="D41" t="n">
-        <v>6710</v>
+        <v>6853</v>
       </c>
       <c r="E41" t="n">
-        <v>1149</v>
+        <v>1159</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-18 11:50 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C2" t="n">
-        <v>9965</v>
+        <v>10987</v>
       </c>
       <c r="D2" t="n">
-        <v>304</v>
+        <v>338</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="F2" t="n">
-        <v>3.57</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>6532</v>
+        <v>7070</v>
       </c>
       <c r="D3" t="n">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="4">
@@ -502,10 +502,10 @@
         <v>34</v>
       </c>
       <c r="C4" t="n">
-        <v>5467</v>
+        <v>5864</v>
       </c>
       <c r="D4" t="n">
-        <v>278</v>
+        <v>300</v>
       </c>
       <c r="E4" t="n">
         <v>26</v>
@@ -524,16 +524,16 @@
         <v>29</v>
       </c>
       <c r="C5" t="n">
-        <v>7362</v>
+        <v>8084</v>
       </c>
       <c r="D5" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E5" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>1.37</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="6">
@@ -543,19 +543,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C6" t="n">
-        <v>5533</v>
+        <v>5879</v>
       </c>
       <c r="D6" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E6" t="n">
         <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>1.77</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C7" t="n">
-        <v>6253</v>
+        <v>6935</v>
       </c>
       <c r="D7" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>0.99</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="8">
@@ -587,10 +587,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3077</v>
+        <v>3119</v>
       </c>
       <c r="D8" t="n">
         <v>138</v>
@@ -599,7 +599,7 @@
         <v>108</v>
       </c>
       <c r="F8" t="n">
-        <v>7.99</v>
+        <v>7.89</v>
       </c>
     </row>
     <row r="9">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>5801</v>
+        <v>6117</v>
       </c>
       <c r="D9" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>2.07</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>3859</v>
+        <v>4311</v>
       </c>
       <c r="D10" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>1.27</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="11">
@@ -656,13 +656,13 @@
         <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>662547</v>
+        <v>666502</v>
       </c>
       <c r="D11" t="n">
-        <v>4061</v>
+        <v>4086</v>
       </c>
       <c r="E11" t="n">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="F11" t="n">
         <v>0.73</v>
@@ -678,16 +678,16 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>5251</v>
+        <v>5339</v>
       </c>
       <c r="D12" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E12" t="n">
         <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>3.39</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="13">
@@ -700,7 +700,7 @@
         <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>8986</v>
+        <v>9032</v>
       </c>
       <c r="D13" t="n">
         <v>172</v>
@@ -709,7 +709,7 @@
         <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1269</v>
+        <v>1277</v>
       </c>
       <c r="D14" t="n">
         <v>10</v>
@@ -731,7 +731,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="15">
@@ -744,16 +744,16 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>3745</v>
+        <v>3771</v>
       </c>
       <c r="D15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="D16" t="n">
         <v>38</v>
@@ -788,82 +788,82 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2050</v>
+        <v>2079</v>
       </c>
       <c r="D17" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E17" t="n">
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.95</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1832</v>
+        <v>803</v>
       </c>
       <c r="D18" t="n">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="E18" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>6.22</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>911</v>
+        <v>1848</v>
       </c>
       <c r="D19" t="n">
-        <v>19</v>
+        <v>100</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F19" t="n">
-        <v>2.2</v>
+        <v>6.28</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>778</v>
+        <v>912</v>
       </c>
       <c r="D20" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3.73</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="D21" t="n">
         <v>14</v>
@@ -885,7 +885,7 @@
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D22" t="n">
         <v>13</v>
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -929,7 +929,7 @@
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>3.19</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="24">
@@ -942,16 +942,16 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>673</v>
+        <v>973</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.59</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="25">
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>627</v>
+        <v>634</v>
       </c>
       <c r="D25" t="n">
         <v>7</v>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="26">
@@ -986,7 +986,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="D26" t="n">
         <v>10</v>
@@ -995,7 +995,7 @@
         <v>7</v>
       </c>
       <c r="F26" t="n">
-        <v>2.92</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="D27" t="n">
         <v>8</v>
@@ -1017,7 +1017,7 @@
         <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>2.26</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="28">
@@ -1052,16 +1052,16 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>5806</v>
+        <v>5973</v>
       </c>
       <c r="D29" t="n">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E29" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F29" t="n">
-        <v>10.73</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="30">
@@ -1096,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>831</v>
+        <v>838</v>
       </c>
       <c r="D31" t="n">
         <v>22</v>
@@ -1105,7 +1105,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.65</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="32">
@@ -1118,16 +1118,16 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="D32" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.6</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="D33" t="n">
         <v>9</v>
@@ -1149,7 +1149,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.97</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="34">
@@ -1184,16 +1184,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>35800</v>
+        <v>55000</v>
       </c>
       <c r="D35" t="n">
-        <v>137</v>
+        <v>186</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>0.39</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="36">
@@ -1206,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
@@ -1228,16 +1228,16 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1194</v>
+        <v>1304</v>
       </c>
       <c r="D37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E37" t="n">
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1272,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D39" t="n">
         <v>4</v>
@@ -1281,7 +1281,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>3.01</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="40">
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
@@ -1303,28 +1303,50 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>xiaomitiengiang.vn</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>98</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>389</v>
-      </c>
-      <c r="C41" t="n">
-        <v>797732</v>
-      </c>
-      <c r="D41" t="n">
-        <v>6853</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1159</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="B42" t="n">
+        <v>403</v>
+      </c>
+      <c r="C42" t="n">
+        <v>826383</v>
+      </c>
+      <c r="D42" t="n">
+        <v>7032</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1186</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-19 11:56 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" t="n">
-        <v>10987</v>
+        <v>11471</v>
       </c>
       <c r="D2" t="n">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="E2" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F2" t="n">
-        <v>3.69</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="3">
@@ -480,60 +480,60 @@
         <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>7070</v>
+        <v>7224</v>
       </c>
       <c r="D3" t="n">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>2.96</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>5864</v>
+        <v>9542</v>
       </c>
       <c r="D4" t="n">
-        <v>300</v>
+        <v>93</v>
       </c>
       <c r="E4" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>5.56</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C5" t="n">
-        <v>8084</v>
+        <v>5928</v>
       </c>
       <c r="D5" t="n">
-        <v>89</v>
+        <v>302</v>
       </c>
       <c r="E5" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>1.36</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="6">
@@ -543,19 +543,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>5879</v>
+        <v>6520</v>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>1.73</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" t="n">
-        <v>6935</v>
+        <v>7992</v>
       </c>
       <c r="D7" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>1.01</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="8">
@@ -590,16 +590,16 @@
         <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3119</v>
+        <v>3234</v>
       </c>
       <c r="D8" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E8" t="n">
         <v>108</v>
       </c>
       <c r="F8" t="n">
-        <v>7.89</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="9">
@@ -612,16 +612,16 @@
         <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>6117</v>
+        <v>6183</v>
       </c>
       <c r="D9" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="10">
@@ -634,16 +634,16 @@
         <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>4311</v>
+        <v>4379</v>
       </c>
       <c r="D10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>1.23</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="11">
@@ -656,13 +656,13 @@
         <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>666502</v>
+        <v>669665</v>
       </c>
       <c r="D11" t="n">
-        <v>4086</v>
+        <v>4107</v>
       </c>
       <c r="E11" t="n">
-        <v>754</v>
+        <v>763</v>
       </c>
       <c r="F11" t="n">
         <v>0.73</v>
@@ -678,7 +678,7 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>5339</v>
+        <v>5401</v>
       </c>
       <c r="D12" t="n">
         <v>160</v>
@@ -687,7 +687,7 @@
         <v>19</v>
       </c>
       <c r="F12" t="n">
-        <v>3.35</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="13">
@@ -700,7 +700,7 @@
         <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>9032</v>
+        <v>9050</v>
       </c>
       <c r="D13" t="n">
         <v>172</v>
@@ -709,7 +709,7 @@
         <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>1277</v>
+        <v>1279</v>
       </c>
       <c r="D14" t="n">
         <v>10</v>
@@ -741,10 +741,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C15" t="n">
-        <v>3771</v>
+        <v>3813</v>
       </c>
       <c r="D15" t="n">
         <v>33</v>
@@ -753,7 +753,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="16">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2079</v>
+        <v>2108</v>
       </c>
       <c r="D17" t="n">
         <v>52</v>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.94</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="18">
@@ -810,126 +810,126 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>803</v>
+        <v>1236</v>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>3.61</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1848</v>
+        <v>634</v>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="E19" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>6.28</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>912</v>
+        <v>1877</v>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>100</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>2.19</v>
+        <v>6.18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>780</v>
+        <v>919</v>
       </c>
       <c r="D21" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.05</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>554</v>
+        <v>799</v>
       </c>
       <c r="D22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.35</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>506</v>
+        <v>554</v>
       </c>
       <c r="D23" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>3.16</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>973</v>
+        <v>991</v>
       </c>
       <c r="D24" t="n">
         <v>7</v>
@@ -951,7 +951,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="25">
@@ -986,7 +986,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="D26" t="n">
         <v>10</v>
@@ -995,7 +995,7 @@
         <v>7</v>
       </c>
       <c r="F26" t="n">
-        <v>2.91</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="D27" t="n">
         <v>8</v>
@@ -1017,7 +1017,7 @@
         <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>2.22</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="28">
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>5973</v>
+        <v>6155</v>
       </c>
       <c r="D29" t="n">
         <v>593</v>
@@ -1061,7 +1061,7 @@
         <v>34</v>
       </c>
       <c r="F29" t="n">
-        <v>10.5</v>
+        <v>10.19</v>
       </c>
     </row>
     <row r="30">
@@ -1096,7 +1096,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="D31" t="n">
         <v>22</v>
@@ -1105,7 +1105,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>2.63</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="32">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="D32" t="n">
         <v>11</v>
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="D33" t="n">
         <v>9</v>
@@ -1149,7 +1149,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>2.86</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="34">
@@ -1184,16 +1184,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>55000</v>
+        <v>73800</v>
       </c>
       <c r="D35" t="n">
-        <v>186</v>
+        <v>237</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="36">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1304</v>
+        <v>1456</v>
       </c>
       <c r="D37" t="n">
         <v>7</v>
@@ -1237,7 +1237,7 @@
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="38">
@@ -1316,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="42">
@@ -1335,16 +1335,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>403</v>
+        <v>420</v>
       </c>
       <c r="C42" t="n">
-        <v>826383</v>
+        <v>853604</v>
       </c>
       <c r="D42" t="n">
-        <v>7032</v>
+        <v>7144</v>
       </c>
       <c r="E42" t="n">
-        <v>1186</v>
+        <v>1204</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-20 13:02 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,13 +458,13 @@
         <v>58</v>
       </c>
       <c r="C2" t="n">
-        <v>11471</v>
+        <v>11627</v>
       </c>
       <c r="D2" t="n">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F2" t="n">
         <v>3.65</v>
@@ -480,16 +480,16 @@
         <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>7224</v>
+        <v>7324</v>
       </c>
       <c r="D3" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>9542</v>
+        <v>9664</v>
       </c>
       <c r="D4" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E4" t="n">
         <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>1.19</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>34</v>
       </c>
       <c r="C5" t="n">
-        <v>5928</v>
+        <v>5998</v>
       </c>
       <c r="D5" t="n">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E5" t="n">
         <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>5.53</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>6520</v>
+        <v>7589</v>
       </c>
       <c r="D6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E6" t="n">
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>1.64</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>27</v>
       </c>
       <c r="C7" t="n">
-        <v>7992</v>
+        <v>8272</v>
       </c>
       <c r="D7" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -590,10 +590,10 @@
         <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3234</v>
+        <v>3248</v>
       </c>
       <c r="D8" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E8" t="n">
         <v>108</v>
@@ -612,16 +612,16 @@
         <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>6183</v>
+        <v>6238</v>
       </c>
       <c r="D9" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="10">
@@ -631,129 +631,129 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" t="n">
-        <v>4379</v>
+        <v>4759</v>
       </c>
       <c r="D10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C11" t="n">
-        <v>669665</v>
+        <v>4446</v>
       </c>
       <c r="D11" t="n">
-        <v>4107</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>763</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>0.73</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>5401</v>
+        <v>673803</v>
       </c>
       <c r="D12" t="n">
-        <v>160</v>
+        <v>4128</v>
       </c>
       <c r="E12" t="n">
-        <v>19</v>
+        <v>765</v>
       </c>
       <c r="F12" t="n">
-        <v>3.31</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>9050</v>
+        <v>5444</v>
       </c>
       <c r="D13" t="n">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>2.03</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9070</v>
+      </c>
+      <c r="D14" t="n">
+        <v>173</v>
+      </c>
+      <c r="E14" t="n">
         <v>12</v>
       </c>
-      <c r="C14" t="n">
-        <v>1279</v>
-      </c>
-      <c r="D14" t="n">
-        <v>10</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
       <c r="F14" t="n">
-        <v>0.78</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>3813</v>
+        <v>1279</v>
       </c>
       <c r="D15" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.97</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="16">
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>1197</v>
+        <v>1569</v>
       </c>
       <c r="D16" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E16" t="n">
         <v>7</v>
       </c>
       <c r="F16" t="n">
-        <v>3.76</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2108</v>
+        <v>2123</v>
       </c>
       <c r="D17" t="n">
         <v>52</v>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.89</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1236</v>
+        <v>1300</v>
       </c>
       <c r="D18" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>2.59</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>634</v>
+        <v>665</v>
       </c>
       <c r="D19" t="n">
         <v>15</v>
@@ -841,7 +841,7 @@
         <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.84</v>
+        <v>2.71</v>
       </c>
     </row>
     <row r="20">
@@ -854,16 +854,16 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>1877</v>
+        <v>1897</v>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E20" t="n">
         <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>6.18</v>
+        <v>6.17</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="D21" t="n">
         <v>20</v>
@@ -885,7 +885,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.29</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>799</v>
+        <v>810</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -907,7 +907,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D23" t="n">
         <v>13</v>
@@ -929,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="24">
@@ -942,16 +942,16 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>991</v>
+        <v>1011</v>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.71</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="25">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D27" t="n">
         <v>8</v>
@@ -1017,139 +1017,139 @@
         <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>43</v>
+        <v>438</v>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>20.93</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>6155</v>
+        <v>43</v>
       </c>
       <c r="D29" t="n">
-        <v>593</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>10.19</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>2852</v>
+        <v>6407</v>
       </c>
       <c r="D30" t="n">
-        <v>33</v>
+        <v>595</v>
       </c>
       <c r="E30" t="n">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>1.68</v>
+        <v>9.82</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>840</v>
+        <v>2852</v>
       </c>
       <c r="D31" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F31" t="n">
-        <v>2.62</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>caothienphat.official</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>762</v>
+        <v>843</v>
       </c>
       <c r="D32" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>1.71</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>caothienphat.official</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>322</v>
+        <v>767</v>
       </c>
       <c r="D33" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>2.8</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="34">
@@ -1184,16 +1184,16 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>73800</v>
+        <v>89800</v>
       </c>
       <c r="D35" t="n">
-        <v>237</v>
+        <v>284</v>
       </c>
       <c r="E35" t="n">
         <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="36">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1456</v>
+        <v>1628</v>
       </c>
       <c r="D37" t="n">
         <v>7</v>
@@ -1237,7 +1237,7 @@
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="38">
@@ -1265,45 +1265,45 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>anhlinhgroup_73</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D39" t="n">
         <v>4</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>2.99</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>bepphuthai</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.75</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="41">
@@ -1316,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="42">
@@ -1335,16 +1335,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="C42" t="n">
-        <v>853604</v>
+        <v>877780</v>
       </c>
       <c r="D42" t="n">
-        <v>7144</v>
+        <v>7265</v>
       </c>
       <c r="E42" t="n">
-        <v>1204</v>
+        <v>1210</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-21 12:31 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C2" t="n">
-        <v>11627</v>
+        <v>12701</v>
       </c>
       <c r="D2" t="n">
-        <v>352</v>
+        <v>369</v>
       </c>
       <c r="E2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F2" t="n">
-        <v>3.65</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="3">
@@ -480,10 +480,10 @@
         <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>7324</v>
+        <v>7387</v>
       </c>
       <c r="D3" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
@@ -502,7 +502,7 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>9664</v>
+        <v>9742</v>
       </c>
       <c r="D4" t="n">
         <v>98</v>
@@ -511,7 +511,7 @@
         <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>34</v>
       </c>
       <c r="C5" t="n">
-        <v>5998</v>
+        <v>6086</v>
       </c>
       <c r="D5" t="n">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="E5" t="n">
         <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>5.5</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>7589</v>
+        <v>7663</v>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E6" t="n">
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" t="n">
-        <v>8272</v>
+        <v>8643</v>
       </c>
       <c r="D7" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="8">
@@ -590,7 +590,7 @@
         <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3248</v>
+        <v>3259</v>
       </c>
       <c r="D8" t="n">
         <v>142</v>
@@ -599,7 +599,7 @@
         <v>108</v>
       </c>
       <c r="F8" t="n">
-        <v>7.7</v>
+        <v>7.67</v>
       </c>
     </row>
     <row r="9">
@@ -612,10 +612,10 @@
         <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>6238</v>
+        <v>6260</v>
       </c>
       <c r="D9" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" t="n">
-        <v>4759</v>
+        <v>4983</v>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>1.22</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="11">
@@ -653,19 +653,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C11" t="n">
-        <v>4446</v>
+        <v>6405</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E11" t="n">
         <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>0.99</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="12">
@@ -678,13 +678,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>673803</v>
+        <v>677660</v>
       </c>
       <c r="D12" t="n">
-        <v>4128</v>
+        <v>4154</v>
       </c>
       <c r="E12" t="n">
-        <v>765</v>
+        <v>773</v>
       </c>
       <c r="F12" t="n">
         <v>0.73</v>
@@ -700,16 +700,16 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5444</v>
+        <v>5489</v>
       </c>
       <c r="D13" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E13" t="n">
         <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>3.29</v>
+        <v>3.28</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>9070</v>
+        <v>9101</v>
       </c>
       <c r="D14" t="n">
         <v>173</v>
@@ -731,7 +731,7 @@
         <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="15">
@@ -766,7 +766,7 @@
         <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>1569</v>
+        <v>1649</v>
       </c>
       <c r="D16" t="n">
         <v>46</v>
@@ -775,7 +775,7 @@
         <v>7</v>
       </c>
       <c r="F16" t="n">
-        <v>3.38</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2123</v>
+        <v>2142</v>
       </c>
       <c r="D17" t="n">
         <v>52</v>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.86</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1300</v>
+        <v>1357</v>
       </c>
       <c r="D18" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E18" t="n">
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>2.77</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>665</v>
+        <v>681</v>
       </c>
       <c r="D19" t="n">
         <v>15</v>
@@ -841,7 +841,7 @@
         <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.71</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="n">
-        <v>1897</v>
+        <v>2027</v>
       </c>
       <c r="D20" t="n">
         <v>101</v>
@@ -863,183 +863,183 @@
         <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>6.17</v>
+        <v>5.77</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>921</v>
+        <v>1270</v>
       </c>
       <c r="D21" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.28</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>810</v>
+        <v>930</v>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1.98</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>555</v>
+        <v>814</v>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>2.34</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>1011</v>
+        <v>585</v>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>0.79</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>634</v>
+        <v>555</v>
       </c>
       <c r="D25" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>1.1</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>587</v>
+        <v>634</v>
       </c>
       <c r="D26" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>2.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>552</v>
+        <v>587</v>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>2.17</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>438</v>
+        <v>558</v>
       </c>
       <c r="D28" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>2.51</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="29">
@@ -1074,16 +1074,16 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>6407</v>
+        <v>6632</v>
       </c>
       <c r="D30" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E30" t="n">
         <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>9.82</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="31">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="D32" t="n">
         <v>22</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1177,176 +1177,198 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>hiephong.techhome</t>
+          <t>hinhnendep7777</t>
         </is>
       </c>
       <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
         <v>1</v>
       </c>
-      <c r="C35" t="n">
-        <v>89800</v>
-      </c>
-      <c r="D35" t="n">
-        <v>284</v>
-      </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>hiephong.techhome</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>2606</v>
+        <v>105400</v>
       </c>
       <c r="D36" t="n">
-        <v>4</v>
+        <v>331</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>0.15</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1628</v>
+        <v>2607</v>
       </c>
       <c r="D37" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0.55</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>roborock.smart.li</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>348</v>
+        <v>1809</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
-        <v>0.29</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>anhlinhgroup_73</t>
+          <t>roborock.smart.li</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>138</v>
+        <v>348</v>
       </c>
       <c r="D39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>3.62</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>bepphuthai</t>
+          <t>anhlinhgroup_73</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="D40" t="n">
         <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>2.99</v>
+        <v>3.52</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>xiaomitiengiang.vn</t>
+          <t>bepphuthai</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0.92</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>xiaomitiengiang.vn</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>112</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.79</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>428</v>
-      </c>
-      <c r="C42" t="n">
-        <v>877780</v>
-      </c>
-      <c r="D42" t="n">
-        <v>7265</v>
-      </c>
-      <c r="E42" t="n">
-        <v>1210</v>
-      </c>
-      <c r="F42" t="inlineStr"/>
+      <c r="B43" t="n">
+        <v>445</v>
+      </c>
+      <c r="C43" t="n">
+        <v>902423</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7396</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1222</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-22 12:41 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C2" t="n">
-        <v>12701</v>
+        <v>13433</v>
       </c>
       <c r="D2" t="n">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="E2" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F2" t="n">
-        <v>3.49</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="3">
@@ -480,16 +480,16 @@
         <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>7387</v>
+        <v>7461</v>
       </c>
       <c r="D3" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>2.96</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="4">
@@ -502,10 +502,10 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>9742</v>
+        <v>9828</v>
       </c>
       <c r="D4" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E4" t="n">
         <v>21</v>
@@ -524,60 +524,60 @@
         <v>34</v>
       </c>
       <c r="C5" t="n">
-        <v>6086</v>
+        <v>6171</v>
       </c>
       <c r="D5" t="n">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="E5" t="n">
         <v>26</v>
       </c>
       <c r="F5" t="n">
-        <v>5.52</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" t="n">
-        <v>7663</v>
+        <v>10436</v>
       </c>
       <c r="D6" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>1.49</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>8643</v>
+        <v>7777</v>
       </c>
       <c r="D7" t="n">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>0.95</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="8">
@@ -590,7 +590,7 @@
         <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3259</v>
+        <v>3266</v>
       </c>
       <c r="D8" t="n">
         <v>142</v>
@@ -599,7 +599,7 @@
         <v>108</v>
       </c>
       <c r="F8" t="n">
-        <v>7.67</v>
+        <v>7.65</v>
       </c>
     </row>
     <row r="9">
@@ -612,7 +612,7 @@
         <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>6260</v>
+        <v>6295</v>
       </c>
       <c r="D9" t="n">
         <v>111</v>
@@ -621,51 +621,51 @@
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C10" t="n">
-        <v>4983</v>
+        <v>6388</v>
       </c>
       <c r="D10" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>1.24</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C11" t="n">
-        <v>6405</v>
+        <v>5358</v>
       </c>
       <c r="D11" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
-        <v>0.84</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="12">
@@ -678,13 +678,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>677660</v>
+        <v>681302</v>
       </c>
       <c r="D12" t="n">
-        <v>4154</v>
+        <v>4171</v>
       </c>
       <c r="E12" t="n">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="F12" t="n">
         <v>0.73</v>
@@ -700,16 +700,16 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5489</v>
+        <v>5532</v>
       </c>
       <c r="D13" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E13" t="n">
         <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>3.28</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="14">
@@ -722,16 +722,16 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>9101</v>
+        <v>9112</v>
       </c>
       <c r="D14" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2080</v>
+      </c>
+      <c r="D16" t="n">
+        <v>54</v>
+      </c>
+      <c r="E16" t="n">
         <v>8</v>
       </c>
-      <c r="C16" t="n">
-        <v>1649</v>
-      </c>
-      <c r="D16" t="n">
-        <v>46</v>
-      </c>
-      <c r="E16" t="n">
-        <v>7</v>
-      </c>
       <c r="F16" t="n">
-        <v>3.21</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="17">
@@ -788,10 +788,10 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2142</v>
+        <v>2168</v>
       </c>
       <c r="D17" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E17" t="n">
         <v>30</v>
@@ -810,7 +810,7 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1357</v>
+        <v>1377</v>
       </c>
       <c r="D18" t="n">
         <v>33</v>
@@ -819,7 +819,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>2.73</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="D19" t="n">
         <v>15</v>
@@ -841,108 +841,108 @@
         <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>2.64</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2027</v>
+        <v>659</v>
       </c>
       <c r="D20" t="n">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>5.77</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>1270</v>
+        <v>2154</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F21" t="n">
-        <v>0.87</v>
+        <v>5.43</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>930</v>
+        <v>1312</v>
       </c>
       <c r="D22" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2.26</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>814</v>
+        <v>932</v>
       </c>
       <c r="D23" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1.97</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>585</v>
+        <v>824</v>
       </c>
       <c r="D24" t="n">
         <v>14</v>
@@ -951,7 +951,7 @@
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>2.74</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="25">
@@ -986,7 +986,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D26" t="n">
         <v>7</v>
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D27" t="n">
         <v>10</v>
@@ -1017,7 +1017,7 @@
         <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>2.9</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="28">
@@ -1030,7 +1030,7 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D28" t="n">
         <v>8</v>
@@ -1039,7 +1039,7 @@
         <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="29">
@@ -1074,16 +1074,16 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>6632</v>
+        <v>6875</v>
       </c>
       <c r="D30" t="n">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="E30" t="n">
         <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>9.5</v>
+        <v>9.220000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="D32" t="n">
         <v>22</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.6</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1184,16 +1184,16 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>8.109999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -1206,16 +1206,16 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>105400</v>
+        <v>122200</v>
       </c>
       <c r="D36" t="n">
-        <v>331</v>
+        <v>396</v>
       </c>
       <c r="E36" t="n">
         <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="37">
@@ -1228,16 +1228,16 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="38">
@@ -1250,16 +1250,16 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>1809</v>
+        <v>2009</v>
       </c>
       <c r="D38" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>
       </c>
       <c r="F38" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="39">
@@ -1294,16 +1294,16 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>3.52</v>
+        <v>4.83</v>
       </c>
     </row>
     <row r="41">
@@ -1316,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D41" t="n">
         <v>4</v>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>2.99</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="42">
@@ -1338,7 +1338,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D42" t="n">
         <v>2</v>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>1.79</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="43">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>445</v>
+        <v>459</v>
       </c>
       <c r="C43" t="n">
-        <v>902423</v>
+        <v>927440</v>
       </c>
       <c r="D43" t="n">
-        <v>7396</v>
+        <v>7555</v>
       </c>
       <c r="E43" t="n">
-        <v>1222</v>
+        <v>1238</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-23 12:38 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C2" t="n">
-        <v>13433</v>
+        <v>13884</v>
       </c>
       <c r="D2" t="n">
-        <v>387</v>
+        <v>401</v>
       </c>
       <c r="E2" t="n">
         <v>83</v>
       </c>
       <c r="F2" t="n">
-        <v>3.5</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="3">
@@ -480,82 +480,82 @@
         <v>36</v>
       </c>
       <c r="C3" t="n">
-        <v>7461</v>
+        <v>7549</v>
       </c>
       <c r="D3" t="n">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>2.95</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>9828</v>
+        <v>11164</v>
       </c>
       <c r="D4" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E4" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>1.22</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C5" t="n">
-        <v>6171</v>
+        <v>9873</v>
       </c>
       <c r="D5" t="n">
-        <v>313</v>
+        <v>99</v>
       </c>
       <c r="E5" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>5.49</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>10436</v>
+        <v>6250</v>
       </c>
       <c r="D6" t="n">
-        <v>93</v>
+        <v>314</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9399999999999999</v>
+        <v>5.44</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>7777</v>
+        <v>7856</v>
       </c>
       <c r="D7" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8">
@@ -590,16 +590,16 @@
         <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3266</v>
+        <v>3286</v>
       </c>
       <c r="D8" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E8" t="n">
         <v>108</v>
       </c>
       <c r="F8" t="n">
-        <v>7.65</v>
+        <v>7.64</v>
       </c>
     </row>
     <row r="9">
@@ -612,60 +612,60 @@
         <v>22</v>
       </c>
       <c r="C9" t="n">
-        <v>6295</v>
+        <v>6341</v>
       </c>
       <c r="D9" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>2.03</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" t="n">
-        <v>6388</v>
+        <v>5674</v>
       </c>
       <c r="D10" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>0.97</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>21</v>
       </c>
       <c r="C11" t="n">
-        <v>5358</v>
+        <v>7792</v>
       </c>
       <c r="D11" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>1.27</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -678,13 +678,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>681302</v>
+        <v>684358</v>
       </c>
       <c r="D12" t="n">
-        <v>4171</v>
+        <v>4190</v>
       </c>
       <c r="E12" t="n">
-        <v>775</v>
+        <v>782</v>
       </c>
       <c r="F12" t="n">
         <v>0.73</v>
@@ -700,7 +700,7 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5532</v>
+        <v>5569</v>
       </c>
       <c r="D13" t="n">
         <v>163</v>
@@ -709,7 +709,7 @@
         <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>3.29</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>9112</v>
+        <v>9123</v>
       </c>
       <c r="D14" t="n">
         <v>174</v>
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>2080</v>
+        <v>2272</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.98</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2168</v>
+        <v>2216</v>
       </c>
       <c r="D17" t="n">
         <v>53</v>
@@ -797,7 +797,7 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.83</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="18">
@@ -810,7 +810,7 @@
         <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1377</v>
+        <v>1382</v>
       </c>
       <c r="D18" t="n">
         <v>33</v>
@@ -819,29 +819,29 @@
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>2.69</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>686</v>
+        <v>894</v>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>2.62</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="20">
@@ -854,104 +854,104 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>659</v>
+        <v>802</v>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>2.58</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>2154</v>
+        <v>689</v>
       </c>
       <c r="D21" t="n">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="E21" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>5.43</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>1312</v>
+        <v>2204</v>
       </c>
       <c r="D22" t="n">
-        <v>13</v>
+        <v>101</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F22" t="n">
-        <v>0.99</v>
+        <v>5.31</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>932</v>
+        <v>1327</v>
       </c>
       <c r="D23" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>2.25</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>824</v>
+        <v>936</v>
       </c>
       <c r="D24" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>1.94</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="25">
@@ -986,7 +986,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="D26" t="n">
         <v>7</v>
@@ -995,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="27">
@@ -1030,7 +1030,7 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="D28" t="n">
         <v>8</v>
@@ -1039,7 +1039,7 @@
         <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>2.14</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="29">
@@ -1074,16 +1074,16 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>6875</v>
+        <v>7076</v>
       </c>
       <c r="D30" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E30" t="n">
         <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>9.220000000000001</v>
+        <v>8.970000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="D32" t="n">
         <v>22</v>
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1149,7 +1149,7 @@
         <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>1.69</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="34">
@@ -1162,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D34" t="n">
         <v>6</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2.13</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="35">
@@ -1184,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>8.109999999999999</v>
+        <v>7.89</v>
       </c>
     </row>
     <row r="36">
@@ -1206,10 +1206,10 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>122200</v>
+        <v>132600</v>
       </c>
       <c r="D36" t="n">
-        <v>396</v>
+        <v>430</v>
       </c>
       <c r="E36" t="n">
         <v>3</v>
@@ -1250,16 +1250,16 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2009</v>
+        <v>2205</v>
       </c>
       <c r="D38" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E38" t="n">
         <v>2</v>
       </c>
       <c r="F38" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="39">
@@ -1294,16 +1294,16 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>4.83</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="41">
@@ -1316,16 +1316,16 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>2.94</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="42">
@@ -1338,7 +1338,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D42" t="n">
         <v>2</v>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>1.77</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="43">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="C43" t="n">
-        <v>927440</v>
+        <v>945155</v>
       </c>
       <c r="D43" t="n">
-        <v>7555</v>
+        <v>7655</v>
       </c>
       <c r="E43" t="n">
-        <v>1238</v>
+        <v>1251</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-24 12:29 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,63 +455,63 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>13884</v>
+        <v>14438</v>
       </c>
       <c r="D2" t="n">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="E2" t="n">
         <v>83</v>
       </c>
       <c r="F2" t="n">
-        <v>3.49</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>.hng0863</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="n">
-        <v>7549</v>
+        <v>11912</v>
       </c>
       <c r="D3" t="n">
-        <v>212</v>
+        <v>103</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>2.94</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>.hng0863</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" t="n">
-        <v>11164</v>
+        <v>7619</v>
       </c>
       <c r="D4" t="n">
-        <v>96</v>
+        <v>218</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="5">
@@ -524,7 +524,7 @@
         <v>35</v>
       </c>
       <c r="C5" t="n">
-        <v>9873</v>
+        <v>9917</v>
       </c>
       <c r="D5" t="n">
         <v>99</v>
@@ -533,7 +533,7 @@
         <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>6250</v>
+        <v>6387</v>
       </c>
       <c r="D6" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E6" t="n">
         <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>5.44</v>
+        <v>5.34</v>
       </c>
     </row>
     <row r="7">
@@ -568,104 +568,104 @@
         <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>7856</v>
+        <v>7932</v>
       </c>
       <c r="D7" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>3286</v>
+        <v>8583</v>
       </c>
       <c r="D8" t="n">
-        <v>143</v>
+        <v>69</v>
       </c>
       <c r="E8" t="n">
-        <v>108</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>7.64</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" t="n">
-        <v>6341</v>
+        <v>5896</v>
       </c>
       <c r="D9" t="n">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="E9" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>2.07</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>5674</v>
+        <v>3300</v>
       </c>
       <c r="D10" t="n">
-        <v>59</v>
+        <v>143</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>108</v>
       </c>
       <c r="F10" t="n">
-        <v>1.2</v>
+        <v>7.61</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>7792</v>
+        <v>6407</v>
       </c>
       <c r="D11" t="n">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F11" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="12">
@@ -678,13 +678,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>684358</v>
+        <v>685904</v>
       </c>
       <c r="D12" t="n">
-        <v>4190</v>
+        <v>4198</v>
       </c>
       <c r="E12" t="n">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="F12" t="n">
         <v>0.73</v>
@@ -700,10 +700,10 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5569</v>
+        <v>5602</v>
       </c>
       <c r="D13" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E13" t="n">
         <v>19</v>
@@ -722,7 +722,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>9123</v>
+        <v>9129</v>
       </c>
       <c r="D14" t="n">
         <v>174</v>
@@ -744,7 +744,7 @@
         <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>1280</v>
+        <v>1283</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
@@ -766,7 +766,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>2272</v>
+        <v>2417</v>
       </c>
       <c r="D16" t="n">
         <v>57</v>
@@ -775,7 +775,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.95</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>2216</v>
+        <v>2250</v>
       </c>
       <c r="D17" t="n">
         <v>53</v>
@@ -797,73 +797,73 @@
         <v>30</v>
       </c>
       <c r="F17" t="n">
-        <v>3.75</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>1382</v>
+        <v>885</v>
       </c>
       <c r="D18" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>2.68</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>894</v>
+        <v>1389</v>
       </c>
       <c r="D19" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>2.01</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>802</v>
+        <v>1019</v>
       </c>
       <c r="D20" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>2.74</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="D21" t="n">
         <v>15</v>
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>2204</v>
+        <v>2213</v>
       </c>
       <c r="D22" t="n">
         <v>101</v>
@@ -907,7 +907,7 @@
         <v>16</v>
       </c>
       <c r="F22" t="n">
-        <v>5.31</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>1327</v>
+        <v>1329</v>
       </c>
       <c r="D23" t="n">
         <v>13</v>
@@ -986,16 +986,16 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D26" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1.09</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="27">
@@ -1030,7 +1030,7 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="D28" t="n">
         <v>8</v>
@@ -1039,7 +1039,7 @@
         <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>2.13</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="29">
@@ -1074,16 +1074,16 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>7076</v>
+        <v>7256</v>
       </c>
       <c r="D30" t="n">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="E30" t="n">
         <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>8.970000000000001</v>
+        <v>8.789999999999999</v>
       </c>
     </row>
     <row r="31">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1149,7 +1149,7 @@
         <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>1.68</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="34">
@@ -1184,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>7.89</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="36">
@@ -1206,16 +1206,16 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>132600</v>
+        <v>142700</v>
       </c>
       <c r="D36" t="n">
-        <v>430</v>
+        <v>447</v>
       </c>
       <c r="E36" t="n">
         <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="37">
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D40" t="n">
         <v>7</v>
@@ -1303,7 +1303,7 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>5.3</v>
+        <v>5.13</v>
       </c>
     </row>
     <row r="41">
@@ -1316,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D41" t="n">
         <v>5</v>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>3.6</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="42">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C43" t="n">
-        <v>945155</v>
+        <v>960163</v>
       </c>
       <c r="D43" t="n">
-        <v>7655</v>
+        <v>7719</v>
       </c>
       <c r="E43" t="n">
-        <v>1251</v>
+        <v>1257</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-25 12:01 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,16 +458,16 @@
         <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>14438</v>
+        <v>14505</v>
       </c>
       <c r="D2" t="n">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="E2" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F2" t="n">
-        <v>3.39</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="3">
@@ -480,10 +480,10 @@
         <v>37</v>
       </c>
       <c r="C3" t="n">
-        <v>11912</v>
+        <v>12069</v>
       </c>
       <c r="D3" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E3" t="n">
         <v>6</v>
@@ -502,16 +502,16 @@
         <v>36</v>
       </c>
       <c r="C4" t="n">
-        <v>7619</v>
+        <v>7694</v>
       </c>
       <c r="D4" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E4" t="n">
         <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>3.01</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="5">
@@ -524,7 +524,7 @@
         <v>35</v>
       </c>
       <c r="C5" t="n">
-        <v>9917</v>
+        <v>9975</v>
       </c>
       <c r="D5" t="n">
         <v>99</v>
@@ -533,7 +533,7 @@
         <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>6387</v>
+        <v>6495</v>
       </c>
       <c r="D6" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E6" t="n">
         <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>5.34</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="7">
@@ -568,16 +568,16 @@
         <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>7932</v>
+        <v>8026</v>
       </c>
       <c r="D7" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="8">
@@ -587,13 +587,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" t="n">
-        <v>8583</v>
+        <v>8996</v>
       </c>
       <c r="D8" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E8" t="n">
         <v>10</v>
@@ -612,16 +612,16 @@
         <v>23</v>
       </c>
       <c r="C9" t="n">
-        <v>5896</v>
+        <v>5991</v>
       </c>
       <c r="D9" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E9" t="n">
         <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>1.2</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
         <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>3300</v>
+        <v>3321</v>
       </c>
       <c r="D10" t="n">
         <v>143</v>
@@ -643,7 +643,7 @@
         <v>108</v>
       </c>
       <c r="F10" t="n">
-        <v>7.61</v>
+        <v>7.56</v>
       </c>
     </row>
     <row r="11">
@@ -656,7 +656,7 @@
         <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>6407</v>
+        <v>6493</v>
       </c>
       <c r="D11" t="n">
         <v>115</v>
@@ -665,7 +665,7 @@
         <v>17</v>
       </c>
       <c r="F11" t="n">
-        <v>2.06</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="12">
@@ -678,10 +678,10 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>685904</v>
+        <v>686934</v>
       </c>
       <c r="D12" t="n">
-        <v>4198</v>
+        <v>4204</v>
       </c>
       <c r="E12" t="n">
         <v>784</v>
@@ -700,16 +700,16 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5602</v>
+        <v>5657</v>
       </c>
       <c r="D13" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E13" t="n">
         <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>3.27</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="14">
@@ -722,7 +722,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>9129</v>
+        <v>9153</v>
       </c>
       <c r="D14" t="n">
         <v>174</v>
@@ -731,7 +731,7 @@
         <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>1283</v>
+        <v>1297</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>2417</v>
+        <v>2430</v>
       </c>
       <c r="D16" t="n">
         <v>57</v>
@@ -775,51 +775,51 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.77</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
-        <v>2250</v>
+        <v>1065</v>
       </c>
       <c r="D17" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="E17" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>3.69</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>885</v>
+        <v>2305</v>
       </c>
       <c r="D18" t="n">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="F18" t="n">
-        <v>2.6</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1389</v>
+        <v>1392</v>
       </c>
       <c r="D19" t="n">
         <v>33</v>
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>1019</v>
+        <v>1032</v>
       </c>
       <c r="D20" t="n">
         <v>18</v>
@@ -863,7 +863,7 @@
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>1.96</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="D21" t="n">
         <v>15</v>
@@ -885,7 +885,7 @@
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>2.61</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>2213</v>
+        <v>2219</v>
       </c>
       <c r="D22" t="n">
         <v>101</v>
@@ -907,7 +907,7 @@
         <v>16</v>
       </c>
       <c r="F22" t="n">
-        <v>5.29</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>1329</v>
+        <v>1340</v>
       </c>
       <c r="D23" t="n">
         <v>13</v>
@@ -929,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="24">
@@ -942,7 +942,7 @@
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="D24" t="n">
         <v>20</v>
@@ -1030,7 +1030,7 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="D28" t="n">
         <v>8</v>
@@ -1039,7 +1039,7 @@
         <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="29">
@@ -1074,16 +1074,16 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>7256</v>
+        <v>7443</v>
       </c>
       <c r="D30" t="n">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="E30" t="n">
         <v>34</v>
       </c>
       <c r="F30" t="n">
-        <v>8.789999999999999</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="31">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="D32" t="n">
         <v>22</v>
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1162,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D34" t="n">
         <v>6</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2.11</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="35">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>2610</v>
+        <v>2611</v>
       </c>
       <c r="D37" t="n">
         <v>5</v>
@@ -1294,16 +1294,16 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>5.13</v>
+        <v>5.56</v>
       </c>
     </row>
     <row r="41">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C43" t="n">
-        <v>960163</v>
+        <v>962952</v>
       </c>
       <c r="D43" t="n">
-        <v>7719</v>
+        <v>7743</v>
       </c>
       <c r="E43" t="n">
-        <v>1257</v>
+        <v>1259</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-26 12:07 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C2" t="n">
-        <v>14505</v>
+        <v>14633</v>
       </c>
       <c r="D2" t="n">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="E2" t="n">
         <v>84</v>
       </c>
       <c r="F2" t="n">
-        <v>3.4</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="3">
@@ -477,63 +477,63 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>12069</v>
+        <v>12498</v>
       </c>
       <c r="D3" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E3" t="n">
         <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>thurobot88</t>
+          <t>momimart.vn</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="n">
-        <v>7694</v>
+        <v>10116</v>
       </c>
       <c r="D4" t="n">
-        <v>219</v>
+        <v>99</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>2.99</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>momimart.vn</t>
+          <t>thurobot88</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" t="n">
-        <v>9975</v>
+        <v>7736</v>
       </c>
       <c r="D5" t="n">
-        <v>99</v>
+        <v>223</v>
       </c>
       <c r="E5" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>1.2</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="6">
@@ -546,7 +546,7 @@
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>6495</v>
+        <v>6561</v>
       </c>
       <c r="D6" t="n">
         <v>316</v>
@@ -555,7 +555,7 @@
         <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>5.27</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="7">
@@ -568,10 +568,10 @@
         <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>8026</v>
+        <v>8086</v>
       </c>
       <c r="D7" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
@@ -590,16 +590,16 @@
         <v>24</v>
       </c>
       <c r="C8" t="n">
-        <v>8996</v>
+        <v>9029</v>
       </c>
       <c r="D8" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E8" t="n">
         <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="9">
@@ -612,16 +612,16 @@
         <v>23</v>
       </c>
       <c r="C9" t="n">
-        <v>5991</v>
+        <v>6047</v>
       </c>
       <c r="D9" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E9" t="n">
         <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
         <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>3321</v>
+        <v>3331</v>
       </c>
       <c r="D10" t="n">
         <v>143</v>
@@ -643,7 +643,7 @@
         <v>108</v>
       </c>
       <c r="F10" t="n">
-        <v>7.56</v>
+        <v>7.54</v>
       </c>
     </row>
     <row r="11">
@@ -656,7 +656,7 @@
         <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>6493</v>
+        <v>6521</v>
       </c>
       <c r="D11" t="n">
         <v>115</v>
@@ -665,7 +665,7 @@
         <v>17</v>
       </c>
       <c r="F11" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="12">
@@ -678,10 +678,10 @@
         <v>14</v>
       </c>
       <c r="C12" t="n">
-        <v>686934</v>
+        <v>688446</v>
       </c>
       <c r="D12" t="n">
-        <v>4204</v>
+        <v>4216</v>
       </c>
       <c r="E12" t="n">
         <v>784</v>
@@ -700,16 +700,16 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5657</v>
+        <v>5729</v>
       </c>
       <c r="D13" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E13" t="n">
         <v>19</v>
       </c>
       <c r="F13" t="n">
-        <v>3.25</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="14">
@@ -722,16 +722,16 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>9153</v>
+        <v>9166</v>
       </c>
       <c r="D14" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="15">
@@ -744,7 +744,7 @@
         <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
@@ -766,7 +766,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>2430</v>
+        <v>2432</v>
       </c>
       <c r="D16" t="n">
         <v>57</v>
@@ -775,7 +775,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.76</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="17">
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>1065</v>
+        <v>11041</v>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>2.25</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>2305</v>
+        <v>2348</v>
       </c>
       <c r="D18" t="n">
         <v>53</v>
       </c>
       <c r="E18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F18" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1392</v>
+        <v>1395</v>
       </c>
       <c r="D19" t="n">
         <v>33</v>
@@ -841,7 +841,7 @@
         <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>2.66</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>1032</v>
+        <v>1036</v>
       </c>
       <c r="D20" t="n">
         <v>18</v>
@@ -863,7 +863,7 @@
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>1.94</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="21">
@@ -898,7 +898,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>2219</v>
+        <v>2225</v>
       </c>
       <c r="D22" t="n">
         <v>101</v>
@@ -907,7 +907,7 @@
         <v>16</v>
       </c>
       <c r="F22" t="n">
-        <v>5.27</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>1340</v>
+        <v>1368</v>
       </c>
       <c r="D23" t="n">
         <v>13</v>
@@ -929,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="24">
@@ -986,7 +986,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D26" t="n">
         <v>8</v>
@@ -1074,16 +1074,16 @@
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>7443</v>
+        <v>7677</v>
       </c>
       <c r="D30" t="n">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="E30" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F30" t="n">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="31">
@@ -1118,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="D32" t="n">
         <v>22</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>2.59</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1149,7 +1149,7 @@
         <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>1.67</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="34">
@@ -1184,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>7.69</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="36">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="D37" t="n">
         <v>5</v>
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D40" t="n">
         <v>8</v>
@@ -1303,7 +1303,7 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>5.56</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="41">
@@ -1316,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D41" t="n">
         <v>5</v>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>3.57</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="42">
@@ -1338,7 +1338,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D42" t="n">
         <v>2</v>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="43">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="C43" t="n">
-        <v>962952</v>
+        <v>975851</v>
       </c>
       <c r="D43" t="n">
-        <v>7743</v>
+        <v>7802</v>
       </c>
       <c r="E43" t="n">
-        <v>1259</v>
+        <v>1262</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
feat: add week 4 winners
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-27 13:46 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,16 +455,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>14633</v>
+        <v>14743</v>
       </c>
       <c r="D2" t="n">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="E2" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F2" t="n">
         <v>3.39</v>
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C3" t="n">
-        <v>12498</v>
+        <v>12884</v>
       </c>
       <c r="D3" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E3" t="n">
         <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="4">
@@ -499,19 +499,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>10116</v>
+        <v>11173</v>
       </c>
       <c r="D4" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E4" t="n">
         <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>1.19</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="5">
@@ -590,16 +590,16 @@
         <v>24</v>
       </c>
       <c r="C8" t="n">
-        <v>9029</v>
+        <v>9076</v>
       </c>
       <c r="D8" t="n">
         <v>74</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C9" t="n">
-        <v>6047</v>
+        <v>6223</v>
       </c>
       <c r="D9" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E9" t="n">
         <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="10">
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>2432</v>
+        <v>2484</v>
       </c>
       <c r="D16" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E16" t="n">
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.75</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="17">
@@ -788,16 +788,16 @@
         <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>11041</v>
+        <v>13250</v>
       </c>
       <c r="D17" t="n">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.48</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="18">
@@ -825,111 +825,111 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1395</v>
+        <v>1582</v>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>2.65</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>1036</v>
+        <v>1395</v>
       </c>
       <c r="D20" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
-        <v>1.93</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>696</v>
+        <v>1042</v>
       </c>
       <c r="D21" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.59</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>2225</v>
+        <v>696</v>
       </c>
       <c r="D22" t="n">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="E22" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>5.26</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>1368</v>
+        <v>2225</v>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>101</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F23" t="n">
-        <v>0.95</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="24">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="C43" t="n">
-        <v>975851</v>
+        <v>980108</v>
       </c>
       <c r="D43" t="n">
-        <v>7802</v>
+        <v>7874</v>
       </c>
       <c r="E43" t="n">
-        <v>1262</v>
+        <v>1265</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-27 14:20 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,7 +458,7 @@
         <v>75</v>
       </c>
       <c r="C2" t="n">
-        <v>14743</v>
+        <v>14775</v>
       </c>
       <c r="D2" t="n">
         <v>415</v>
@@ -467,7 +467,7 @@
         <v>85</v>
       </c>
       <c r="F2" t="n">
-        <v>3.39</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="3">
@@ -480,7 +480,7 @@
         <v>42</v>
       </c>
       <c r="C3" t="n">
-        <v>12884</v>
+        <v>13072</v>
       </c>
       <c r="D3" t="n">
         <v>113</v>
@@ -489,7 +489,7 @@
         <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="4">
@@ -502,7 +502,7 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>11173</v>
+        <v>11179</v>
       </c>
       <c r="D4" t="n">
         <v>104</v>
@@ -590,7 +590,7 @@
         <v>24</v>
       </c>
       <c r="C8" t="n">
-        <v>9076</v>
+        <v>9078</v>
       </c>
       <c r="D8" t="n">
         <v>74</v>
@@ -612,7 +612,7 @@
         <v>24</v>
       </c>
       <c r="C9" t="n">
-        <v>6223</v>
+        <v>6225</v>
       </c>
       <c r="D9" t="n">
         <v>70</v>
@@ -627,45 +627,45 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>nc.nh.qu.robot</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>3331</v>
+        <v>6527</v>
       </c>
       <c r="D10" t="n">
-        <v>143</v>
+        <v>115</v>
       </c>
       <c r="E10" t="n">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="F10" t="n">
-        <v>7.54</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>nc.nh.qu.robot</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" t="n">
-        <v>6521</v>
+        <v>3331</v>
       </c>
       <c r="D11" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="E11" t="n">
-        <v>17</v>
+        <v>108</v>
       </c>
       <c r="F11" t="n">
-        <v>2.02</v>
+        <v>7.54</v>
       </c>
     </row>
     <row r="12">
@@ -766,7 +766,7 @@
         <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>2484</v>
+        <v>2499</v>
       </c>
       <c r="D16" t="n">
         <v>62</v>
@@ -775,7 +775,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="17">
@@ -788,16 +788,16 @@
         <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>13250</v>
+        <v>13274</v>
       </c>
       <c r="D17" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="18">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1582</v>
+        <v>1585</v>
       </c>
       <c r="D19" t="n">
         <v>15</v>
@@ -957,67 +957,67 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>555</v>
+        <v>598</v>
       </c>
       <c r="D25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
-        <v>2.34</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>642</v>
+        <v>555</v>
       </c>
       <c r="D26" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1.25</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>588</v>
+        <v>642</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>2.89</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="28">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C43" t="n">
-        <v>980108</v>
+        <v>980396</v>
       </c>
       <c r="D43" t="n">
-        <v>7874</v>
+        <v>7877</v>
       </c>
       <c r="E43" t="n">
         <v>1265</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-28 12:30 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C2" t="n">
-        <v>14775</v>
+        <v>15212</v>
       </c>
       <c r="D2" t="n">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="E2" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" t="n">
-        <v>3.38</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C3" t="n">
-        <v>13072</v>
+        <v>14918</v>
       </c>
       <c r="D3" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E3" t="n">
         <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>0.91</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="4">
@@ -502,7 +502,7 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>11179</v>
+        <v>11199</v>
       </c>
       <c r="D4" t="n">
         <v>104</v>
@@ -521,19 +521,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" t="n">
-        <v>7736</v>
+        <v>7909</v>
       </c>
       <c r="D5" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E5" t="n">
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>3.02</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="6">
@@ -587,63 +587,63 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C8" t="n">
-        <v>9078</v>
+        <v>10364</v>
       </c>
       <c r="D8" t="n">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>robothutbuiductrong</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" t="n">
-        <v>6225</v>
+        <v>7306</v>
       </c>
       <c r="D9" t="n">
-        <v>70</v>
+        <v>119</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>1.27</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>robothutbuiductrong</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" t="n">
-        <v>6527</v>
+        <v>6272</v>
       </c>
       <c r="D10" t="n">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="E10" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>2.02</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="11">
@@ -766,16 +766,16 @@
         <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>2499</v>
+        <v>2607</v>
       </c>
       <c r="D16" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E16" t="n">
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.88</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="17">
@@ -788,16 +788,16 @@
         <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>13274</v>
+        <v>13550</v>
       </c>
       <c r="D17" t="n">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="18">
@@ -832,7 +832,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1585</v>
+        <v>1587</v>
       </c>
       <c r="D19" t="n">
         <v>15</v>
@@ -876,16 +876,16 @@
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="D21" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>1.92</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -935,45 +935,45 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>937</v>
+        <v>977</v>
       </c>
       <c r="D24" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>2.24</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>598</v>
+        <v>937</v>
       </c>
       <c r="D25" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>3.01</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="26">
@@ -1184,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>7.5</v>
+        <v>7.14</v>
       </c>
     </row>
     <row r="36">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>492</v>
+        <v>505</v>
       </c>
       <c r="C43" t="n">
-        <v>980396</v>
+        <v>985757</v>
       </c>
       <c r="D43" t="n">
-        <v>7877</v>
+        <v>7928</v>
       </c>
       <c r="E43" t="n">
-        <v>1265</v>
+        <v>1269</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-29 12:41 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C2" t="n">
-        <v>15212</v>
+        <v>15568</v>
       </c>
       <c r="D2" t="n">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="E2" t="n">
         <v>86</v>
       </c>
       <c r="F2" t="n">
-        <v>3.34</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C3" t="n">
-        <v>14918</v>
+        <v>15497</v>
       </c>
       <c r="D3" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="4">
@@ -502,10 +502,10 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>11199</v>
+        <v>11209</v>
       </c>
       <c r="D4" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E4" t="n">
         <v>21</v>
@@ -524,16 +524,16 @@
         <v>37</v>
       </c>
       <c r="C5" t="n">
-        <v>7909</v>
+        <v>7923</v>
       </c>
       <c r="D5" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E5" t="n">
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>2.97</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="6">
@@ -587,19 +587,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>10364</v>
+        <v>10723</v>
       </c>
       <c r="D8" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="9">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C9" t="n">
-        <v>7306</v>
+        <v>7988</v>
       </c>
       <c r="D9" t="n">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>1.86</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C10" t="n">
-        <v>6272</v>
+        <v>6405</v>
       </c>
       <c r="D10" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="11">
@@ -766,7 +766,7 @@
         <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>2607</v>
+        <v>2617</v>
       </c>
       <c r="D16" t="n">
         <v>64</v>
@@ -775,7 +775,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="17">
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C17" t="n">
-        <v>13550</v>
+        <v>13703</v>
       </c>
       <c r="D17" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="18">
@@ -825,133 +825,133 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>1587</v>
+        <v>2331</v>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>102</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F19" t="n">
-        <v>0.95</v>
+        <v>5.06</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>1395</v>
+        <v>1588</v>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>2.65</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1048</v>
+        <v>1395</v>
       </c>
       <c r="D21" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>696</v>
+        <v>1124</v>
       </c>
       <c r="D22" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
-        <v>2.59</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>2225</v>
+        <v>1059</v>
       </c>
       <c r="D23" t="n">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="E23" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>5.26</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24" t="n">
-        <v>977</v>
+        <v>696</v>
       </c>
       <c r="D24" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>2.05</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="25">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>505</v>
+        <v>518</v>
       </c>
       <c r="C43" t="n">
-        <v>985757</v>
+        <v>988318</v>
       </c>
       <c r="D43" t="n">
-        <v>7928</v>
+        <v>7967</v>
       </c>
       <c r="E43" t="n">
-        <v>1269</v>
+        <v>1273</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-30 12:25 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C2" t="n">
-        <v>15568</v>
+        <v>16398</v>
       </c>
       <c r="D2" t="n">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="E2" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F2" t="n">
-        <v>3.3</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C3" t="n">
-        <v>15497</v>
+        <v>16267</v>
       </c>
       <c r="D3" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>11209</v>
+        <v>11224</v>
       </c>
       <c r="D4" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E4" t="n">
         <v>21</v>
       </c>
       <c r="F4" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>37</v>
       </c>
       <c r="C5" t="n">
-        <v>7923</v>
+        <v>7930</v>
       </c>
       <c r="D5" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E5" t="n">
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="6">
@@ -561,45 +561,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7" t="n">
-        <v>8086</v>
+        <v>11959</v>
       </c>
       <c r="D7" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>1.52</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="n">
-        <v>10723</v>
+        <v>8086</v>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="E8" t="n">
         <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>0.99</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="9">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" t="n">
-        <v>7988</v>
+        <v>8828</v>
       </c>
       <c r="D9" t="n">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E9" t="n">
         <v>17</v>
       </c>
       <c r="F9" t="n">
-        <v>1.85</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="10">
@@ -634,10 +634,10 @@
         <v>26</v>
       </c>
       <c r="C10" t="n">
-        <v>6405</v>
+        <v>6472</v>
       </c>
       <c r="D10" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -737,45 +737,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>1298</v>
+        <v>2771</v>
       </c>
       <c r="D15" t="n">
+        <v>68</v>
+      </c>
+      <c r="E15" t="n">
         <v>10</v>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
       <c r="F15" t="n">
-        <v>0.77</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>2617</v>
+        <v>1298</v>
       </c>
       <c r="D16" t="n">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>2.83</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="17">
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>13703</v>
+        <v>15401</v>
       </c>
       <c r="D17" t="n">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="18">
@@ -825,177 +825,177 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>2331</v>
+        <v>799</v>
       </c>
       <c r="D19" t="n">
-        <v>102</v>
+        <v>16</v>
       </c>
       <c r="E19" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>5.06</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>1588</v>
+        <v>2340</v>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>102</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>0.9399999999999999</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1395</v>
+        <v>1588</v>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.65</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>1124</v>
+        <v>1395</v>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>1.87</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1059</v>
+        <v>1131</v>
       </c>
       <c r="D23" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.98</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>5</v>
       </c>
       <c r="C24" t="n">
-        <v>696</v>
+        <v>1067</v>
       </c>
       <c r="D24" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>2.59</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>domotekvietnam</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>937</v>
+        <v>637</v>
       </c>
       <c r="D25" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.24</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>domotekvietnam</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>555</v>
+        <v>937</v>
       </c>
       <c r="D26" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2.34</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="27">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>518</v>
+        <v>532</v>
       </c>
       <c r="C43" t="n">
-        <v>988318</v>
+        <v>994144</v>
       </c>
       <c r="D43" t="n">
-        <v>7967</v>
+        <v>8027</v>
       </c>
       <c r="E43" t="n">
-        <v>1273</v>
+        <v>1278</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-07-31 12:38 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C2" t="n">
-        <v>16398</v>
+        <v>17466</v>
       </c>
       <c r="D2" t="n">
-        <v>442</v>
+        <v>464</v>
       </c>
       <c r="E2" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F2" t="n">
-        <v>3.24</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C3" t="n">
-        <v>16267</v>
+        <v>16656</v>
       </c>
       <c r="D3" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="4">
@@ -499,10 +499,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11224</v>
+        <v>11279</v>
       </c>
       <c r="D4" t="n">
         <v>106</v>
@@ -524,7 +524,7 @@
         <v>37</v>
       </c>
       <c r="C5" t="n">
-        <v>7930</v>
+        <v>7934</v>
       </c>
       <c r="D5" t="n">
         <v>226</v>
@@ -568,10 +568,10 @@
         <v>33</v>
       </c>
       <c r="C7" t="n">
-        <v>11959</v>
+        <v>12125</v>
       </c>
       <c r="D7" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
@@ -583,45 +583,45 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>thietbibepan</t>
+          <t>xiaomi.phu.tho</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>8086</v>
+        <v>9165</v>
       </c>
       <c r="D8" t="n">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="E8" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>1.52</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>xiaomi.phu.tho</t>
+          <t>thietbibepan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" t="n">
-        <v>8828</v>
+        <v>8086</v>
       </c>
       <c r="D9" t="n">
-        <v>139</v>
+        <v>108</v>
       </c>
       <c r="E9" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9" t="n">
-        <v>1.77</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="10">
@@ -634,7 +634,7 @@
         <v>26</v>
       </c>
       <c r="C10" t="n">
-        <v>6472</v>
+        <v>6474</v>
       </c>
       <c r="D10" t="n">
         <v>74</v>
@@ -741,19 +741,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>2771</v>
+        <v>3201</v>
       </c>
       <c r="D15" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
-        <v>2.81</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="16">
@@ -788,7 +788,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15401</v>
+        <v>15504</v>
       </c>
       <c r="D17" t="n">
         <v>132</v>
@@ -797,7 +797,7 @@
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="18">
@@ -832,16 +832,16 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="D19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.38</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2340</v>
+        <v>2349</v>
       </c>
       <c r="D20" t="n">
         <v>102</v>
@@ -863,7 +863,7 @@
         <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>5.04</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="21">
@@ -920,7 +920,7 @@
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1131</v>
+        <v>1133</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -929,7 +929,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.86</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="24">
@@ -964,16 +964,16 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>637</v>
+        <v>726</v>
       </c>
       <c r="D25" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.35</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="26">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>532</v>
+        <v>540</v>
       </c>
       <c r="C43" t="n">
-        <v>994144</v>
+        <v>996802</v>
       </c>
       <c r="D43" t="n">
-        <v>8027</v>
+        <v>8071</v>
       </c>
       <c r="E43" t="n">
-        <v>1278</v>
+        <v>1285</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-01 11:56 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>17466</v>
+        <v>17909</v>
       </c>
       <c r="D2" t="n">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="E2" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F2" t="n">
-        <v>3.19</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="3">
@@ -480,10 +480,10 @@
         <v>49</v>
       </c>
       <c r="C3" t="n">
-        <v>16656</v>
+        <v>16690</v>
       </c>
       <c r="D3" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
@@ -502,16 +502,16 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11279</v>
+        <v>11587</v>
       </c>
       <c r="D4" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" t="n">
-        <v>1.13</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="5">
@@ -521,63 +521,63 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>7934</v>
+        <v>8055</v>
       </c>
       <c r="D5" t="n">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E5" t="n">
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>2.99</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>kimanh_1202</t>
+          <t>3t.smart.robot.tn</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>6561</v>
+        <v>12498</v>
       </c>
       <c r="D6" t="n">
-        <v>316</v>
+        <v>109</v>
       </c>
       <c r="E6" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>5.21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3t.smart.robot.tn</t>
+          <t>kimanh_1202</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" t="n">
-        <v>12125</v>
+        <v>6561</v>
       </c>
       <c r="D7" t="n">
-        <v>106</v>
+        <v>316</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="8">
@@ -590,10 +590,10 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9165</v>
+        <v>9247</v>
       </c>
       <c r="D8" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E8" t="n">
         <v>17</v>
@@ -634,7 +634,7 @@
         <v>26</v>
       </c>
       <c r="C10" t="n">
-        <v>6474</v>
+        <v>6476</v>
       </c>
       <c r="D10" t="n">
         <v>74</v>
@@ -715,45 +715,45 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>9166</v>
+        <v>3311</v>
       </c>
       <c r="D14" t="n">
-        <v>175</v>
+        <v>86</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>2.04</v>
+        <v>2.93</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>3201</v>
+        <v>9166</v>
       </c>
       <c r="D15" t="n">
-        <v>78</v>
+        <v>175</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F15" t="n">
-        <v>2.78</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="16">
@@ -788,7 +788,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15504</v>
+        <v>15512</v>
       </c>
       <c r="D17" t="n">
         <v>132</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="D20" t="n">
         <v>102</v>
@@ -920,7 +920,7 @@
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>726</v>
+        <v>739</v>
       </c>
       <c r="D25" t="n">
         <v>16</v>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.2</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="26">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="C43" t="n">
-        <v>996802</v>
+        <v>998303</v>
       </c>
       <c r="D43" t="n">
-        <v>8071</v>
+        <v>8094</v>
       </c>
       <c r="E43" t="n">
-        <v>1285</v>
+        <v>1290</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-02 11:52 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,16 +458,16 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>17909</v>
+        <v>17956</v>
       </c>
       <c r="D2" t="n">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E2" t="n">
         <v>97</v>
       </c>
       <c r="F2" t="n">
-        <v>3.17</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="3">
@@ -480,7 +480,7 @@
         <v>49</v>
       </c>
       <c r="C3" t="n">
-        <v>16690</v>
+        <v>16719</v>
       </c>
       <c r="D3" t="n">
         <v>132</v>
@@ -502,16 +502,16 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11587</v>
+        <v>11599</v>
       </c>
       <c r="D4" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E4" t="n">
         <v>22</v>
       </c>
       <c r="F4" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8055</v>
+        <v>8080</v>
       </c>
       <c r="D5" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E5" t="n">
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>2.97</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>12498</v>
+        <v>12525</v>
       </c>
       <c r="D6" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="7">
@@ -590,7 +590,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9247</v>
+        <v>9292</v>
       </c>
       <c r="D8" t="n">
         <v>145</v>
@@ -599,7 +599,7 @@
         <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>1.75</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="9">
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" t="n">
         <v>6476</v>
@@ -722,7 +722,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>3311</v>
+        <v>3344</v>
       </c>
       <c r="D14" t="n">
         <v>86</v>
@@ -731,7 +731,7 @@
         <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15512</v>
+        <v>15516</v>
       </c>
       <c r="D17" t="n">
         <v>132</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -841,7 +841,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.74</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2352</v>
+        <v>2363</v>
       </c>
       <c r="D20" t="n">
         <v>102</v>
@@ -863,7 +863,7 @@
         <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>5.02</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="21">
@@ -920,7 +920,7 @@
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="D25" t="n">
         <v>16</v>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.17</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="26">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C43" t="n">
-        <v>998303</v>
+        <v>998546</v>
       </c>
       <c r="D43" t="n">
-        <v>8094</v>
+        <v>8100</v>
       </c>
       <c r="E43" t="n">
         <v>1290</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-03 13:40 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,10 +458,10 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>17956</v>
+        <v>18018</v>
       </c>
       <c r="D2" t="n">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E2" t="n">
         <v>97</v>
@@ -480,7 +480,7 @@
         <v>49</v>
       </c>
       <c r="C3" t="n">
-        <v>16719</v>
+        <v>16756</v>
       </c>
       <c r="D3" t="n">
         <v>132</v>
@@ -502,7 +502,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11599</v>
+        <v>11604</v>
       </c>
       <c r="D4" t="n">
         <v>108</v>
@@ -524,16 +524,16 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8080</v>
+        <v>8083</v>
       </c>
       <c r="D5" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E5" t="n">
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="6">
@@ -543,19 +543,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>12525</v>
+        <v>12907</v>
       </c>
       <c r="D6" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="7">
@@ -590,16 +590,16 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9292</v>
+        <v>9321</v>
       </c>
       <c r="D8" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E8" t="n">
         <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="9">
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>6476</v>
+        <v>6483</v>
       </c>
       <c r="D10" t="n">
         <v>74</v>
@@ -722,16 +722,16 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>3344</v>
+        <v>3360</v>
       </c>
       <c r="D14" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E14" t="n">
         <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>2.9</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15516</v>
+        <v>15520</v>
       </c>
       <c r="D17" t="n">
         <v>132</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -841,7 +841,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.73</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2363</v>
+        <v>2364</v>
       </c>
       <c r="D20" t="n">
         <v>102</v>
@@ -920,7 +920,7 @@
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="D23" t="n">
         <v>14</v>
@@ -929,7 +929,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.85</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="24">
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D25" t="n">
         <v>16</v>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="26">
@@ -1001,133 +1001,133 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>642</v>
+        <v>979</v>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>1.25</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>569</v>
+        <v>642</v>
       </c>
       <c r="D28" t="n">
         <v>8</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>2.11</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>43</v>
+        <v>569</v>
       </c>
       <c r="D29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
-        <v>20.93</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>7677</v>
+        <v>43</v>
       </c>
       <c r="D30" t="n">
-        <v>609</v>
+        <v>9</v>
       </c>
       <c r="E30" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>8.4</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>saigonbephcm</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>2852</v>
+        <v>7677</v>
       </c>
       <c r="D31" t="n">
-        <v>33</v>
+        <v>609</v>
       </c>
       <c r="E31" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="F31" t="n">
-        <v>1.68</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>saigonbephcm</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>852</v>
+        <v>2852</v>
       </c>
       <c r="D32" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>2.58</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="33">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C43" t="n">
-        <v>998546</v>
+        <v>999225</v>
       </c>
       <c r="D43" t="n">
-        <v>8100</v>
+        <v>8106</v>
       </c>
       <c r="E43" t="n">
         <v>1290</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-03 14:25 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,7 +458,7 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18018</v>
+        <v>18019</v>
       </c>
       <c r="D2" t="n">
         <v>472</v>
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>979</v>
+        <v>982</v>
       </c>
       <c r="D27" t="n">
         <v>23</v>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>2.35</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="28">
@@ -1360,7 +1360,7 @@
         <v>548</v>
       </c>
       <c r="C43" t="n">
-        <v>999225</v>
+        <v>999229</v>
       </c>
       <c r="D43" t="n">
         <v>8106</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-04 12:39 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,7 +458,7 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18019</v>
+        <v>18034</v>
       </c>
       <c r="D2" t="n">
         <v>472</v>
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>16756</v>
+        <v>16992</v>
       </c>
       <c r="D3" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="4">
@@ -502,7 +502,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11604</v>
+        <v>11611</v>
       </c>
       <c r="D4" t="n">
         <v>108</v>
@@ -524,7 +524,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8083</v>
+        <v>8086</v>
       </c>
       <c r="D5" t="n">
         <v>232</v>
@@ -546,16 +546,16 @@
         <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>12907</v>
+        <v>12919</v>
       </c>
       <c r="D6" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="7">
@@ -590,7 +590,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9321</v>
+        <v>9336</v>
       </c>
       <c r="D8" t="n">
         <v>146</v>
@@ -634,7 +634,7 @@
         <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>6483</v>
+        <v>6485</v>
       </c>
       <c r="D10" t="n">
         <v>74</v>
@@ -722,16 +722,16 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>3360</v>
+        <v>3364</v>
       </c>
       <c r="D14" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>2.92</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15520</v>
+        <v>15535</v>
       </c>
       <c r="D17" t="n">
         <v>132</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -854,7 +854,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2364</v>
+        <v>2366</v>
       </c>
       <c r="D20" t="n">
         <v>102</v>
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="D25" t="n">
         <v>16</v>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.14</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="26">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>982</v>
+        <v>1004</v>
       </c>
       <c r="D27" t="n">
         <v>23</v>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>2.34</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="28">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C43" t="n">
-        <v>999229</v>
+        <v>999568</v>
       </c>
       <c r="D43" t="n">
-        <v>8106</v>
+        <v>8111</v>
       </c>
       <c r="E43" t="n">
-        <v>1290</v>
+        <v>1293</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-05 12:36 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,10 +458,10 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18034</v>
+        <v>18064</v>
       </c>
       <c r="D2" t="n">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E2" t="n">
         <v>97</v>
@@ -480,10 +480,10 @@
         <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>16992</v>
+        <v>17142</v>
       </c>
       <c r="D3" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
@@ -502,7 +502,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11611</v>
+        <v>11615</v>
       </c>
       <c r="D4" t="n">
         <v>108</v>
@@ -524,7 +524,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8086</v>
+        <v>8087</v>
       </c>
       <c r="D5" t="n">
         <v>232</v>
@@ -533,7 +533,7 @@
         <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>3.01</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -546,7 +546,7 @@
         <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>12919</v>
+        <v>12933</v>
       </c>
       <c r="D6" t="n">
         <v>112</v>
@@ -590,10 +590,10 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9336</v>
+        <v>9365</v>
       </c>
       <c r="D8" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E8" t="n">
         <v>17</v>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="n">
         <v>6485</v>
@@ -671,67 +671,67 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>688446</v>
+        <v>3406</v>
       </c>
       <c r="D12" t="n">
-        <v>4216</v>
+        <v>91</v>
       </c>
       <c r="E12" t="n">
-        <v>784</v>
+        <v>15</v>
       </c>
       <c r="F12" t="n">
-        <v>0.73</v>
+        <v>3.11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>5729</v>
+        <v>688446</v>
       </c>
       <c r="D13" t="n">
-        <v>166</v>
+        <v>4216</v>
       </c>
       <c r="E13" t="n">
-        <v>19</v>
+        <v>784</v>
       </c>
       <c r="F13" t="n">
-        <v>3.23</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>3364</v>
+        <v>5729</v>
       </c>
       <c r="D14" t="n">
-        <v>90</v>
+        <v>166</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F14" t="n">
-        <v>3.09</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="15">
@@ -788,16 +788,16 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15535</v>
+        <v>15538</v>
       </c>
       <c r="D17" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="18">
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -841,7 +841,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.72</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="20">
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="D25" t="n">
         <v>16</v>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="26">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>1004</v>
+        <v>1013</v>
       </c>
       <c r="D27" t="n">
         <v>23</v>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="28">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="C43" t="n">
-        <v>999568</v>
+        <v>999861</v>
       </c>
       <c r="D43" t="n">
-        <v>8111</v>
+        <v>8116</v>
       </c>
       <c r="E43" t="n">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
chore(report): update qrevo dashboard data
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,16 +458,16 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18064</v>
+        <v>18230</v>
       </c>
       <c r="D2" t="n">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="E2" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F2" t="n">
-        <v>3.16</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" t="n">
-        <v>17142</v>
+        <v>17773</v>
       </c>
       <c r="D3" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="4">
@@ -502,16 +502,16 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11615</v>
+        <v>11799</v>
       </c>
       <c r="D4" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F4" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="5">
@@ -524,16 +524,16 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8087</v>
+        <v>8564</v>
       </c>
       <c r="D5" t="n">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="6">
@@ -546,16 +546,16 @@
         <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>12933</v>
+        <v>13100</v>
       </c>
       <c r="D6" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7" t="n">
-        <v>6561</v>
+        <v>7259</v>
       </c>
       <c r="D7" t="n">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="E7" t="n">
         <v>26</v>
       </c>
       <c r="F7" t="n">
-        <v>5.21</v>
+        <v>4.88</v>
       </c>
     </row>
     <row r="8">
@@ -590,16 +590,16 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9365</v>
+        <v>9710</v>
       </c>
       <c r="D8" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F8" t="n">
-        <v>1.75</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="9">
@@ -612,16 +612,16 @@
         <v>31</v>
       </c>
       <c r="C9" t="n">
-        <v>8086</v>
+        <v>8184</v>
       </c>
       <c r="D9" t="n">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="E9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>1.52</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>6485</v>
+        <v>6913</v>
       </c>
       <c r="D10" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="11">
@@ -656,16 +656,16 @@
         <v>23</v>
       </c>
       <c r="C11" t="n">
-        <v>3331</v>
+        <v>3261</v>
       </c>
       <c r="D11" t="n">
         <v>143</v>
       </c>
       <c r="E11" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F11" t="n">
-        <v>7.54</v>
+        <v>7.67</v>
       </c>
     </row>
     <row r="12">
@@ -678,16 +678,16 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>3406</v>
+        <v>3634</v>
       </c>
       <c r="D12" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E12" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F12" t="n">
-        <v>3.11</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="13">
@@ -700,13 +700,13 @@
         <v>14</v>
       </c>
       <c r="C13" t="n">
-        <v>688446</v>
+        <v>700602</v>
       </c>
       <c r="D13" t="n">
-        <v>4216</v>
+        <v>4291</v>
       </c>
       <c r="E13" t="n">
-        <v>784</v>
+        <v>812</v>
       </c>
       <c r="F13" t="n">
         <v>0.73</v>
@@ -722,16 +722,16 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>5729</v>
+        <v>5761</v>
       </c>
       <c r="D14" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E14" t="n">
         <v>19</v>
       </c>
       <c r="F14" t="n">
-        <v>3.23</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="15">
@@ -744,16 +744,16 @@
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>9166</v>
+        <v>10079</v>
       </c>
       <c r="D15" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="E15" t="n">
         <v>12</v>
       </c>
       <c r="F15" t="n">
-        <v>2.04</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="16">
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>1298</v>
+        <v>1296</v>
       </c>
       <c r="D16" t="n">
         <v>10</v>
@@ -788,16 +788,16 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>15538</v>
+        <v>15678</v>
       </c>
       <c r="D17" t="n">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="E17" t="n">
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="18">
@@ -810,16 +810,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>2348</v>
+        <v>2684</v>
       </c>
       <c r="D18" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E18" t="n">
         <v>32</v>
       </c>
       <c r="F18" t="n">
-        <v>3.62</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>816</v>
+        <v>825</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -841,7 +841,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.7</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="20">
@@ -854,16 +854,16 @@
         <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2366</v>
+        <v>2368</v>
       </c>
       <c r="D20" t="n">
         <v>102</v>
       </c>
       <c r="E20" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F20" t="n">
-        <v>4.99</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="21">
@@ -876,16 +876,16 @@
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1588</v>
+        <v>1603</v>
       </c>
       <c r="D21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="22">
@@ -898,7 +898,7 @@
         <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>1395</v>
+        <v>1407</v>
       </c>
       <c r="D22" t="n">
         <v>33</v>
@@ -907,51 +907,51 @@
         <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>2.65</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1139</v>
+        <v>1223</v>
       </c>
       <c r="D23" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>1.84</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>5</v>
       </c>
       <c r="C24" t="n">
-        <v>1067</v>
+        <v>1144</v>
       </c>
       <c r="D24" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>1.97</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="25">
@@ -964,16 +964,16 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="D25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.11</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="26">
@@ -986,16 +986,16 @@
         <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>937</v>
+        <v>928</v>
       </c>
       <c r="D26" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2.24</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>1013</v>
+        <v>1032</v>
       </c>
       <c r="D27" t="n">
         <v>23</v>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>2.27</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="28">
@@ -1030,16 +1030,16 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>642</v>
+        <v>687</v>
       </c>
       <c r="D28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>1.25</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="29">
@@ -1052,7 +1052,7 @@
         <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>569</v>
+        <v>533</v>
       </c>
       <c r="D29" t="n">
         <v>8</v>
@@ -1061,7 +1061,7 @@
         <v>4</v>
       </c>
       <c r="F29" t="n">
-        <v>2.11</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="30">
@@ -1096,16 +1096,16 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>7677</v>
+        <v>5621</v>
       </c>
       <c r="D31" t="n">
-        <v>609</v>
+        <v>589</v>
       </c>
       <c r="E31" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F31" t="n">
-        <v>8.4</v>
+        <v>11.01</v>
       </c>
     </row>
     <row r="32">
@@ -1118,16 +1118,16 @@
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>2852</v>
+        <v>3642</v>
       </c>
       <c r="D32" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E32" t="n">
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>1.68</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="33">
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>784</v>
+        <v>809</v>
       </c>
       <c r="D33" t="n">
         <v>11</v>
@@ -1149,7 +1149,7 @@
         <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>1.66</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="34">
@@ -1162,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>287</v>
+        <v>361</v>
       </c>
       <c r="D34" t="n">
         <v>6</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2.09</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="35">
@@ -1184,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D35" t="n">
         <v>3</v>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>7.14</v>
+        <v>7.32</v>
       </c>
     </row>
     <row r="36">
@@ -1206,60 +1206,60 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>142700</v>
+        <v>193200</v>
       </c>
       <c r="D36" t="n">
-        <v>447</v>
+        <v>555</v>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F36" t="n">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>t_tech.ninhbinh</t>
+          <t>thietbithongminh8</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>2613</v>
+        <v>6150</v>
       </c>
       <c r="D37" t="n">
+        <v>26</v>
+      </c>
+      <c r="E37" t="n">
         <v>5</v>
       </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
       <c r="F37" t="n">
-        <v>0.19</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>thietbithongminh8</t>
+          <t>t_tech.ninhbinh</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2205</v>
+        <v>2613</v>
       </c>
       <c r="D38" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.59</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="39">
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D40" t="n">
         <v>8</v>
@@ -1303,7 +1303,7 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>5.52</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="41">
@@ -1316,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D41" t="n">
         <v>5</v>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>3.55</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="42">
@@ -1338,7 +1338,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D42" t="n">
         <v>2</v>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>1.71</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="43">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C43" t="n">
-        <v>999861</v>
+        <v>1070298</v>
       </c>
       <c r="D43" t="n">
-        <v>8116</v>
+        <v>8367</v>
       </c>
       <c r="E43" t="n">
-        <v>1294</v>
+        <v>1330</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-06 12:40 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +458,7 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18230</v>
+        <v>18234</v>
       </c>
       <c r="D2" t="n">
         <v>477</v>
@@ -524,7 +524,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8564</v>
+        <v>8565</v>
       </c>
       <c r="D5" t="n">
         <v>237</v>
@@ -546,7 +546,7 @@
         <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>13100</v>
+        <v>13101</v>
       </c>
       <c r="D6" t="n">
         <v>113</v>
@@ -590,7 +590,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9710</v>
+        <v>9715</v>
       </c>
       <c r="D8" t="n">
         <v>149</v>
@@ -785,10 +785,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>15678</v>
+        <v>15741</v>
       </c>
       <c r="D17" t="n">
         <v>146</v>
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="D25" t="n">
         <v>17</v>
@@ -1357,10 +1357,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C43" t="n">
-        <v>1070298</v>
+        <v>1070373</v>
       </c>
       <c r="D43" t="n">
         <v>8367</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-07 11:23 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,7 +458,7 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18234</v>
+        <v>18236</v>
       </c>
       <c r="D2" t="n">
         <v>477</v>
@@ -480,7 +480,7 @@
         <v>51</v>
       </c>
       <c r="C3" t="n">
-        <v>17773</v>
+        <v>17775</v>
       </c>
       <c r="D3" t="n">
         <v>143</v>
@@ -502,7 +502,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="n">
-        <v>11799</v>
+        <v>11803</v>
       </c>
       <c r="D4" t="n">
         <v>110</v>
@@ -524,7 +524,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8565</v>
+        <v>8568</v>
       </c>
       <c r="D5" t="n">
         <v>237</v>
@@ -546,7 +546,7 @@
         <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>13101</v>
+        <v>13102</v>
       </c>
       <c r="D6" t="n">
         <v>113</v>
@@ -590,7 +590,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="n">
-        <v>9715</v>
+        <v>9717</v>
       </c>
       <c r="D8" t="n">
         <v>149</v>
@@ -634,7 +634,7 @@
         <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>6913</v>
+        <v>6919</v>
       </c>
       <c r="D10" t="n">
         <v>77</v>
@@ -678,7 +678,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>3634</v>
+        <v>3637</v>
       </c>
       <c r="D12" t="n">
         <v>94</v>
@@ -788,7 +788,7 @@
         <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>15741</v>
+        <v>15790</v>
       </c>
       <c r="D17" t="n">
         <v>146</v>
@@ -797,7 +797,7 @@
         <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -825,67 +825,67 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>825</v>
+        <v>1978</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>2.67</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>825</v>
+      </c>
+      <c r="D20" t="n">
+        <v>17</v>
+      </c>
+      <c r="E20" t="n">
         <v>5</v>
       </c>
-      <c r="C20" t="n">
-        <v>2368</v>
-      </c>
-      <c r="D20" t="n">
-        <v>102</v>
-      </c>
-      <c r="E20" t="n">
-        <v>17</v>
-      </c>
       <c r="F20" t="n">
-        <v>5.03</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1603</v>
+        <v>2368</v>
       </c>
       <c r="D21" t="n">
-        <v>14</v>
+        <v>102</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F21" t="n">
-        <v>0.87</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="22">
@@ -1008,16 +1008,16 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="D27" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>2.23</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="28">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C43" t="n">
-        <v>1070373</v>
+        <v>1070821</v>
       </c>
       <c r="D43" t="n">
-        <v>8367</v>
+        <v>8371</v>
       </c>
       <c r="E43" t="n">
         <v>1330</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-08 11:12 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -458,7 +458,7 @@
         <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>18236</v>
+        <v>18237</v>
       </c>
       <c r="D2" t="n">
         <v>477</v>
@@ -524,7 +524,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>8568</v>
+        <v>8570</v>
       </c>
       <c r="D5" t="n">
         <v>237</v>
@@ -788,7 +788,7 @@
         <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>15790</v>
+        <v>15792</v>
       </c>
       <c r="D17" t="n">
         <v>146</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>1978</v>
+        <v>1986</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -1360,7 +1360,7 @@
         <v>556</v>
       </c>
       <c r="C43" t="n">
-        <v>1070821</v>
+        <v>1070834</v>
       </c>
       <c r="D43" t="n">
         <v>8371</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-09 11:11 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -477,13 +477,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" t="n">
-        <v>17775</v>
+        <v>18156</v>
       </c>
       <c r="D3" t="n">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
@@ -546,7 +546,7 @@
         <v>35</v>
       </c>
       <c r="C6" t="n">
-        <v>13102</v>
+        <v>13105</v>
       </c>
       <c r="D6" t="n">
         <v>113</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>1986</v>
+        <v>1991</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -841,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="20">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C43" t="n">
-        <v>1070834</v>
+        <v>1071223</v>
       </c>
       <c r="D43" t="n">
-        <v>8371</v>
+        <v>8374</v>
       </c>
       <c r="E43" t="n">
         <v>1330</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-10 11:40 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -480,7 +480,7 @@
         <v>52</v>
       </c>
       <c r="C3" t="n">
-        <v>18156</v>
+        <v>18176</v>
       </c>
       <c r="D3" t="n">
         <v>146</v>
@@ -678,7 +678,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>3637</v>
+        <v>3638</v>
       </c>
       <c r="D12" t="n">
         <v>94</v>
@@ -788,7 +788,7 @@
         <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>15792</v>
+        <v>15793</v>
       </c>
       <c r="D17" t="n">
         <v>146</v>
@@ -825,67 +825,67 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>1991</v>
+        <v>2483</v>
       </c>
       <c r="D19" t="n">
-        <v>17</v>
+        <v>106</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F19" t="n">
-        <v>0.85</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>825</v>
+        <v>1993</v>
       </c>
       <c r="D20" t="n">
         <v>17</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>2.67</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>825</v>
+      </c>
+      <c r="D21" t="n">
+        <v>17</v>
+      </c>
+      <c r="E21" t="n">
         <v>5</v>
       </c>
-      <c r="C21" t="n">
-        <v>2368</v>
-      </c>
-      <c r="D21" t="n">
-        <v>102</v>
-      </c>
-      <c r="E21" t="n">
-        <v>17</v>
-      </c>
       <c r="F21" t="n">
-        <v>5.03</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="22">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C43" t="n">
-        <v>1071223</v>
+        <v>1071362</v>
       </c>
       <c r="D43" t="n">
-        <v>8374</v>
+        <v>8378</v>
       </c>
       <c r="E43" t="n">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-10 12:49 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -678,7 +678,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>3638</v>
+        <v>3639</v>
       </c>
       <c r="D12" t="n">
         <v>94</v>
@@ -832,7 +832,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>2483</v>
+        <v>2484</v>
       </c>
       <c r="D19" t="n">
         <v>106</v>
@@ -1360,7 +1360,7 @@
         <v>558</v>
       </c>
       <c r="C43" t="n">
-        <v>1071362</v>
+        <v>1071364</v>
       </c>
       <c r="D43" t="n">
         <v>8378</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-11 11:24 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -788,7 +788,7 @@
         <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>15793</v>
+        <v>15794</v>
       </c>
       <c r="D17" t="n">
         <v>146</v>
@@ -803,45 +803,45 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>2684</v>
+        <v>2619</v>
       </c>
       <c r="D18" t="n">
-        <v>54</v>
+        <v>108</v>
       </c>
       <c r="E18" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F18" t="n">
-        <v>3.2</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>2484</v>
+        <v>2684</v>
       </c>
       <c r="D19" t="n">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="E19" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F19" t="n">
-        <v>4.99</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>1993</v>
+        <v>1997</v>
       </c>
       <c r="D20" t="n">
         <v>17</v>
@@ -1001,111 +1001,111 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tm.anh.kitchen.qu</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>1033</v>
+        <v>5666</v>
       </c>
       <c r="D27" t="n">
-        <v>24</v>
+        <v>590</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>2.32</v>
+        <v>10.94</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>nhadepbepxinh.camxuyen</t>
+          <t>tm.anh.kitchen.qu</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>687</v>
+        <v>1033</v>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>1.31</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>giangchismarthome</t>
+          <t>nhadepbepxinh.camxuyen</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>533</v>
+        <v>687</v>
       </c>
       <c r="D29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2.25</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>roborockthanhhoa</t>
+          <t>giangchismarthome</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>43</v>
+        <v>533</v>
       </c>
       <c r="D30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F30" t="n">
-        <v>20.93</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>roborockthanhhoa</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>5621</v>
+        <v>43</v>
       </c>
       <c r="D31" t="n">
-        <v>589</v>
+        <v>9</v>
       </c>
       <c r="E31" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>11.01</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="32">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C43" t="n">
-        <v>1071364</v>
+        <v>1071549</v>
       </c>
       <c r="D43" t="n">
-        <v>8378</v>
+        <v>8381</v>
       </c>
       <c r="E43" t="n">
         <v>1331</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-12 11:32 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -678,7 +678,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>3639</v>
+        <v>3641</v>
       </c>
       <c r="D12" t="n">
         <v>94</v>
@@ -759,89 +759,89 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>mistorebienhoa</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>1296</v>
+        <v>15945</v>
       </c>
       <c r="D16" t="n">
-        <v>10</v>
+        <v>147</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>0.77</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>mistorebienhoa</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>15794</v>
+        <v>1296</v>
       </c>
       <c r="D17" t="n">
-        <v>146</v>
+        <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>2619</v>
+        <v>3139</v>
       </c>
       <c r="D18" t="n">
-        <v>108</v>
+        <v>57</v>
       </c>
       <c r="E18" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F18" t="n">
-        <v>4.81</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="E19" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F19" t="n">
-        <v>3.2</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="D20" t="n">
         <v>17</v>
@@ -869,67 +869,67 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>825</v>
+        <v>1395</v>
       </c>
       <c r="D21" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.67</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="n">
+        <v>825</v>
+      </c>
+      <c r="D22" t="n">
+        <v>17</v>
+      </c>
+      <c r="E22" t="n">
         <v>5</v>
       </c>
-      <c r="C22" t="n">
-        <v>1407</v>
-      </c>
-      <c r="D22" t="n">
-        <v>33</v>
-      </c>
-      <c r="E22" t="n">
-        <v>4</v>
-      </c>
       <c r="F22" t="n">
-        <v>2.63</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1223</v>
+        <v>1407</v>
       </c>
       <c r="D23" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>1.88</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="24">
@@ -1008,16 +1008,16 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5666</v>
+        <v>5798</v>
       </c>
       <c r="D27" t="n">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="E27" t="n">
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>10.94</v>
+        <v>10.76</v>
       </c>
     </row>
     <row r="28">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C43" t="n">
-        <v>1071549</v>
+        <v>1072665</v>
       </c>
       <c r="D43" t="n">
-        <v>8381</v>
+        <v>8409</v>
       </c>
       <c r="E43" t="n">
         <v>1331</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-13 11:30 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>15945</v>
+        <v>15995</v>
       </c>
       <c r="D16" t="n">
         <v>147</v>
@@ -810,16 +810,16 @@
         <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>3139</v>
+        <v>3220</v>
       </c>
       <c r="D18" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E18" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F18" t="n">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>2821</v>
+        <v>2837</v>
       </c>
       <c r="D19" t="n">
         <v>116</v>
@@ -841,7 +841,7 @@
         <v>18</v>
       </c>
       <c r="F19" t="n">
-        <v>4.75</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="20">
@@ -851,19 +851,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>1999</v>
+        <v>2360</v>
       </c>
       <c r="D20" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.85</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="21">
@@ -876,16 +876,16 @@
         <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>1395</v>
+        <v>1475</v>
       </c>
       <c r="D21" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.51</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="22">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5798</v>
+        <v>5810</v>
       </c>
       <c r="D27" t="n">
         <v>594</v>
@@ -1017,7 +1017,7 @@
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>10.76</v>
+        <v>10.74</v>
       </c>
     </row>
     <row r="28">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C43" t="n">
-        <v>1072665</v>
+        <v>1073265</v>
       </c>
       <c r="D43" t="n">
-        <v>8409</v>
+        <v>8412</v>
       </c>
       <c r="E43" t="n">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-14 11:29 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -480,7 +480,7 @@
         <v>52</v>
       </c>
       <c r="C3" t="n">
-        <v>18176</v>
+        <v>18177</v>
       </c>
       <c r="D3" t="n">
         <v>146</v>
@@ -543,13 +543,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="n">
-        <v>13105</v>
+        <v>13239</v>
       </c>
       <c r="D6" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>15995</v>
+        <v>16008</v>
       </c>
       <c r="D16" t="n">
         <v>147</v>
@@ -810,7 +810,7 @@
         <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>3220</v>
+        <v>3229</v>
       </c>
       <c r="D18" t="n">
         <v>58</v>
@@ -819,7 +819,7 @@
         <v>33</v>
       </c>
       <c r="F18" t="n">
-        <v>2.83</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="19">
@@ -832,16 +832,16 @@
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>2837</v>
+        <v>2857</v>
       </c>
       <c r="D19" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E19" t="n">
         <v>18</v>
       </c>
       <c r="F19" t="n">
-        <v>4.72</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2360</v>
+        <v>2365</v>
       </c>
       <c r="D20" t="n">
         <v>18</v>
@@ -876,7 +876,7 @@
         <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>1475</v>
+        <v>1495</v>
       </c>
       <c r="D21" t="n">
         <v>34</v>
@@ -885,73 +885,73 @@
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>2.44</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>825</v>
+        <v>1407</v>
       </c>
       <c r="D22" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>2.67</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1407</v>
+        <v>1305</v>
       </c>
       <c r="D23" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>2.63</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="n">
+        <v>825</v>
+      </c>
+      <c r="D24" t="n">
+        <v>17</v>
+      </c>
+      <c r="E24" t="n">
         <v>5</v>
       </c>
-      <c r="C24" t="n">
-        <v>1144</v>
-      </c>
-      <c r="D24" t="n">
-        <v>14</v>
-      </c>
-      <c r="E24" t="n">
-        <v>7</v>
-      </c>
       <c r="F24" t="n">
-        <v>1.84</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="25">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5810</v>
+        <v>5813</v>
       </c>
       <c r="D27" t="n">
         <v>594</v>
@@ -1017,7 +1017,7 @@
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>10.74</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="28">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="C43" t="n">
-        <v>1073265</v>
+        <v>1073631</v>
       </c>
       <c r="D43" t="n">
-        <v>8412</v>
+        <v>8416</v>
       </c>
       <c r="E43" t="n">
         <v>1332</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-15 10:59 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -543,19 +543,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="n">
-        <v>13239</v>
+        <v>13991</v>
       </c>
       <c r="D6" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="7">
@@ -766,10 +766,10 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>16008</v>
+        <v>16016</v>
       </c>
       <c r="D16" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -803,111 +803,111 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>3229</v>
+        <v>2058</v>
       </c>
       <c r="D18" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E18" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
-        <v>2.82</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>2857</v>
+        <v>3242</v>
       </c>
       <c r="D19" t="n">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="E19" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F19" t="n">
-        <v>4.73</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2365</v>
+        <v>2868</v>
       </c>
       <c r="D20" t="n">
+        <v>117</v>
+      </c>
+      <c r="E20" t="n">
         <v>18</v>
       </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
       <c r="F20" t="n">
-        <v>0.76</v>
+        <v>4.71</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>1495</v>
+        <v>2367</v>
       </c>
       <c r="D21" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.41</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>1407</v>
+        <v>1504</v>
       </c>
       <c r="D22" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.63</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1305</v>
+        <v>1331</v>
       </c>
       <c r="D23" t="n">
         <v>16</v>
@@ -929,7 +929,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.76</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="24">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5813</v>
+        <v>5817</v>
       </c>
       <c r="D27" t="n">
         <v>594</v>
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="C43" t="n">
-        <v>1073631</v>
+        <v>1075107</v>
       </c>
       <c r="D43" t="n">
-        <v>8416</v>
+        <v>8428</v>
       </c>
       <c r="E43" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-16 10:58 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -546,10 +546,10 @@
         <v>37</v>
       </c>
       <c r="C6" t="n">
-        <v>13991</v>
+        <v>14014</v>
       </c>
       <c r="D6" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>16016</v>
+        <v>16021</v>
       </c>
       <c r="D16" t="n">
         <v>148</v>
@@ -810,16 +810,16 @@
         <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>2058</v>
+        <v>3022</v>
       </c>
       <c r="D18" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>2.19</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="19">
@@ -832,16 +832,16 @@
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>3242</v>
+        <v>3245</v>
       </c>
       <c r="D19" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E19" t="n">
         <v>33</v>
       </c>
       <c r="F19" t="n">
-        <v>2.81</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2868</v>
+        <v>2881</v>
       </c>
       <c r="D20" t="n">
         <v>117</v>
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="F20" t="n">
-        <v>4.71</v>
+        <v>4.69</v>
       </c>
     </row>
     <row r="21">
@@ -898,16 +898,16 @@
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>1504</v>
+        <v>1538</v>
       </c>
       <c r="D22" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.39</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1331</v>
+        <v>1334</v>
       </c>
       <c r="D23" t="n">
         <v>16</v>
@@ -929,7 +929,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="24">
@@ -1008,16 +1008,16 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5817</v>
+        <v>5829</v>
       </c>
       <c r="D27" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E27" t="n">
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>10.73</v>
+        <v>10.72</v>
       </c>
     </row>
     <row r="28">
@@ -1360,13 +1360,13 @@
         <v>573</v>
       </c>
       <c r="C43" t="n">
-        <v>1075107</v>
+        <v>1076164</v>
       </c>
       <c r="D43" t="n">
-        <v>8428</v>
+        <v>8443</v>
       </c>
       <c r="E43" t="n">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-17 11:08 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -546,7 +546,7 @@
         <v>37</v>
       </c>
       <c r="C6" t="n">
-        <v>14014</v>
+        <v>14020</v>
       </c>
       <c r="D6" t="n">
         <v>119</v>
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>16021</v>
+        <v>16025</v>
       </c>
       <c r="D16" t="n">
         <v>148</v>
@@ -810,16 +810,16 @@
         <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>3022</v>
+        <v>3044</v>
       </c>
       <c r="D18" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E18" t="n">
         <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>1.85</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="19">
@@ -832,7 +832,7 @@
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>3245</v>
+        <v>3252</v>
       </c>
       <c r="D19" t="n">
         <v>59</v>
@@ -841,7 +841,7 @@
         <v>33</v>
       </c>
       <c r="F19" t="n">
-        <v>2.84</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2881</v>
+        <v>2887</v>
       </c>
       <c r="D20" t="n">
         <v>117</v>
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="F20" t="n">
-        <v>4.69</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="21">
@@ -876,7 +876,7 @@
         <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>2367</v>
+        <v>2368</v>
       </c>
       <c r="D21" t="n">
         <v>18</v>
@@ -898,7 +898,7 @@
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>1538</v>
+        <v>1570</v>
       </c>
       <c r="D22" t="n">
         <v>36</v>
@@ -907,7 +907,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.47</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1334</v>
+        <v>1342</v>
       </c>
       <c r="D23" t="n">
         <v>16</v>
@@ -929,7 +929,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="24">
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5829</v>
+        <v>5836</v>
       </c>
       <c r="D27" t="n">
         <v>595</v>
@@ -1017,7 +1017,7 @@
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>10.72</v>
+        <v>10.71</v>
       </c>
     </row>
     <row r="28">
@@ -1360,10 +1360,10 @@
         <v>573</v>
       </c>
       <c r="C43" t="n">
-        <v>1076164</v>
+        <v>1076257</v>
       </c>
       <c r="D43" t="n">
-        <v>8443</v>
+        <v>8445</v>
       </c>
       <c r="E43" t="n">
         <v>1334</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-17 12:19 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>6919</v>
+        <v>6930</v>
       </c>
       <c r="D10" t="n">
         <v>77</v>
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>16025</v>
+        <v>16029</v>
       </c>
       <c r="D16" t="n">
         <v>148</v>
@@ -810,7 +810,7 @@
         <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>3044</v>
+        <v>3045</v>
       </c>
       <c r="D18" t="n">
         <v>52</v>
@@ -819,7 +819,7 @@
         <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>1.91</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="19">
@@ -854,7 +854,7 @@
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2887</v>
+        <v>2888</v>
       </c>
       <c r="D20" t="n">
         <v>117</v>
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="F20" t="n">
-        <v>4.68</v>
+        <v>4.67</v>
       </c>
     </row>
     <row r="21">
@@ -898,7 +898,7 @@
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>1570</v>
+        <v>1572</v>
       </c>
       <c r="D22" t="n">
         <v>36</v>
@@ -1357,10 +1357,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C43" t="n">
-        <v>1076257</v>
+        <v>1076276</v>
       </c>
       <c r="D43" t="n">
         <v>8445</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-18 11:10 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -546,16 +546,16 @@
         <v>37</v>
       </c>
       <c r="C6" t="n">
-        <v>14020</v>
+        <v>14024</v>
       </c>
       <c r="D6" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E6" t="n">
         <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="7">
@@ -634,16 +634,16 @@
         <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>6930</v>
+        <v>7153</v>
       </c>
       <c r="D10" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>1.24</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="11">
@@ -766,7 +766,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>16029</v>
+        <v>16037</v>
       </c>
       <c r="D16" t="n">
         <v>148</v>
@@ -781,45 +781,45 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>homecaredigital</t>
+          <t>thuyduonggiadung</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>1296</v>
+        <v>3211</v>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>0.77</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>thuyduonggiadung</t>
+          <t>homecaredigital</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C18" t="n">
-        <v>3045</v>
+        <v>1296</v>
       </c>
       <c r="D18" t="n">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>1.9</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="19">
@@ -832,16 +832,16 @@
         <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>3252</v>
+        <v>3262</v>
       </c>
       <c r="D19" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
         <v>33</v>
       </c>
       <c r="F19" t="n">
-        <v>2.83</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="20">
@@ -854,7 +854,7 @@
         <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2888</v>
+        <v>2900</v>
       </c>
       <c r="D20" t="n">
         <v>117</v>
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="F20" t="n">
-        <v>4.67</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="21">
@@ -898,7 +898,7 @@
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>1572</v>
+        <v>1593</v>
       </c>
       <c r="D22" t="n">
         <v>36</v>
@@ -907,7 +907,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>2.42</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="23">
@@ -920,7 +920,7 @@
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="D23" t="n">
         <v>16</v>
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>5836</v>
+        <v>5844</v>
       </c>
       <c r="D27" t="n">
         <v>595</v>
@@ -1017,7 +1017,7 @@
         <v>30</v>
       </c>
       <c r="F27" t="n">
-        <v>10.71</v>
+        <v>10.69</v>
       </c>
     </row>
     <row r="28">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C43" t="n">
-        <v>1076276</v>
+        <v>1076730</v>
       </c>
       <c r="D43" t="n">
-        <v>8445</v>
+        <v>8452</v>
       </c>
       <c r="E43" t="n">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-20 10:48 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -546,7 +546,7 @@
         <v>37</v>
       </c>
       <c r="C6" t="n">
-        <v>14024</v>
+        <v>14028</v>
       </c>
       <c r="D6" t="n">
         <v>120</v>
@@ -634,7 +634,7 @@
         <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>7153</v>
+        <v>7187</v>
       </c>
       <c r="D10" t="n">
         <v>79</v>
@@ -643,7 +643,7 @@
         <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="11">
@@ -788,7 +788,7 @@
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>3211</v>
+        <v>3400</v>
       </c>
       <c r="D17" t="n">
         <v>55</v>
@@ -797,7 +797,7 @@
         <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>1.93</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="18">
@@ -920,16 +920,16 @@
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1344</v>
+        <v>1351</v>
       </c>
       <c r="D23" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E23" t="n">
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1.71</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="24">
@@ -1360,10 +1360,10 @@
         <v>575</v>
       </c>
       <c r="C43" t="n">
-        <v>1076730</v>
+        <v>1076964</v>
       </c>
       <c r="D43" t="n">
-        <v>8452</v>
+        <v>8454</v>
       </c>
       <c r="E43" t="n">
         <v>1335</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-21 10:50 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -546,7 +546,7 @@
         <v>37</v>
       </c>
       <c r="C6" t="n">
-        <v>14028</v>
+        <v>14032</v>
       </c>
       <c r="D6" t="n">
         <v>120</v>
@@ -788,7 +788,7 @@
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>3400</v>
+        <v>3408</v>
       </c>
       <c r="D17" t="n">
         <v>55</v>
@@ -1360,7 +1360,7 @@
         <v>575</v>
       </c>
       <c r="C43" t="n">
-        <v>1076964</v>
+        <v>1076976</v>
       </c>
       <c r="D43" t="n">
         <v>8454</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-22 10:43 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -634,7 +634,7 @@
         <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>7187</v>
+        <v>7191</v>
       </c>
       <c r="D10" t="n">
         <v>79</v>
@@ -788,7 +788,7 @@
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>3408</v>
+        <v>3410</v>
       </c>
       <c r="D17" t="n">
         <v>55</v>
@@ -1360,7 +1360,7 @@
         <v>575</v>
       </c>
       <c r="C43" t="n">
-        <v>1076976</v>
+        <v>1076982</v>
       </c>
       <c r="D43" t="n">
         <v>8454</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-23 10:50 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -634,16 +634,16 @@
         <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>7191</v>
+        <v>7195</v>
       </c>
       <c r="D10" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>1.22</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="11">
@@ -715,45 +715,45 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bothome_robotgialai</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>5761</v>
+        <v>10469</v>
       </c>
       <c r="D14" t="n">
-        <v>165</v>
+        <v>187</v>
       </c>
       <c r="E14" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>3.19</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>bothome_robotgialai</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>10079</v>
+        <v>5761</v>
       </c>
       <c r="D15" t="n">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F15" t="n">
-        <v>1.9</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="16">
@@ -788,16 +788,16 @@
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>3410</v>
+        <v>3411</v>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E17" t="n">
         <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>1.82</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="18">
@@ -1357,16 +1357,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C43" t="n">
-        <v>1076982</v>
+        <v>1077377</v>
       </c>
       <c r="D43" t="n">
-        <v>8454</v>
+        <v>8463</v>
       </c>
       <c r="E43" t="n">
-        <v>1335</v>
+        <v>1337</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-24 11:14 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -634,7 +634,7 @@
         <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>7195</v>
+        <v>7196</v>
       </c>
       <c r="D10" t="n">
         <v>80</v>
@@ -722,7 +722,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>10469</v>
+        <v>10478</v>
       </c>
       <c r="D14" t="n">
         <v>187</v>
@@ -788,16 +788,16 @@
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>3411</v>
+        <v>3412</v>
       </c>
       <c r="D17" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17" t="n">
         <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>1.85</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="18">
@@ -1360,10 +1360,10 @@
         <v>576</v>
       </c>
       <c r="C43" t="n">
-        <v>1077377</v>
+        <v>1077388</v>
       </c>
       <c r="D43" t="n">
-        <v>8463</v>
+        <v>8464</v>
       </c>
       <c r="E43" t="n">
         <v>1337</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-24 12:26 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C3" t="n">
-        <v>18177</v>
+        <v>18569</v>
       </c>
       <c r="D3" t="n">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="4">
@@ -722,16 +722,16 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>10478</v>
+        <v>10480</v>
       </c>
       <c r="D14" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E14" t="n">
         <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>1.92</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="15">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C43" t="n">
-        <v>1077388</v>
+        <v>1077782</v>
       </c>
       <c r="D43" t="n">
-        <v>8464</v>
+        <v>8471</v>
       </c>
       <c r="E43" t="n">
         <v>1337</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-08-25 11:03 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -480,7 +480,7 @@
         <v>53</v>
       </c>
       <c r="C3" t="n">
-        <v>18569</v>
+        <v>18570</v>
       </c>
       <c r="D3" t="n">
         <v>152</v>
@@ -722,7 +722,7 @@
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>10480</v>
+        <v>10493</v>
       </c>
       <c r="D14" t="n">
         <v>188</v>
@@ -788,7 +788,7 @@
         <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>3412</v>
+        <v>3414</v>
       </c>
       <c r="D17" t="n">
         <v>57</v>
@@ -797,7 +797,7 @@
         <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>1.88</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="18">
@@ -1360,7 +1360,7 @@
         <v>577</v>
       </c>
       <c r="C43" t="n">
-        <v>1077782</v>
+        <v>1077798</v>
       </c>
       <c r="D43" t="n">
         <v>8471</v>

</xml_diff>

<commit_message>
update qrevo videos + report (2026-09-09 14:58 UTC)
</commit_message>
<xml_diff>
--- a/output/qrevo-summary.xlsx
+++ b/output/qrevo-summary.xlsx
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C3" t="n">
-        <v>18570</v>
+        <v>18721</v>
       </c>
       <c r="D3" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="4">
@@ -521,19 +521,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="n">
-        <v>8570</v>
+        <v>8791</v>
       </c>
       <c r="D5" t="n">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E5" t="n">
         <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>2.99</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="6">
@@ -587,19 +587,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" t="n">
-        <v>9717</v>
+        <v>10166</v>
       </c>
       <c r="D8" t="n">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="E8" t="n">
         <v>18</v>
       </c>
       <c r="F8" t="n">
-        <v>1.72</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="9">
@@ -671,67 +671,67 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tigerbot.smarthome</t>
+          <t>mivietnam_chuyengiarobot</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>3641</v>
+        <v>10990</v>
       </c>
       <c r="D12" t="n">
-        <v>94</v>
+        <v>198</v>
       </c>
       <c r="E12" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F12" t="n">
-        <v>3.05</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>minhchautestthat</t>
+          <t>tigerbot.smarthome</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" t="n">
-        <v>700602</v>
+        <v>3641</v>
       </c>
       <c r="D13" t="n">
-        <v>4291</v>
+        <v>94</v>
       </c>
       <c r="E13" t="n">
-        <v>812</v>
+        <v>17</v>
       </c>
       <c r="F13" t="n">
-        <v>0.73</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>mivietnam_chuyengiarobot</t>
+          <t>minhchautestthat</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>14</v>
       </c>
       <c r="C14" t="n">
-        <v>10493</v>
+        <v>700602</v>
       </c>
       <c r="D14" t="n">
-        <v>188</v>
+        <v>4291</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>812</v>
       </c>
       <c r="F14" t="n">
-        <v>1.93</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="15">
@@ -825,133 +825,133 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>quyrobot</t>
+          <t>homebotvietnam</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C19" t="n">
-        <v>3262</v>
+        <v>3049</v>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E19" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>2.85</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>roborock.krng.n</t>
+          <t>quyrobot</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C20" t="n">
-        <v>2900</v>
+        <v>3902</v>
       </c>
       <c r="D20" t="n">
-        <v>117</v>
+        <v>65</v>
       </c>
       <c r="E20" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F20" t="n">
-        <v>4.66</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>homebotvietnam</t>
+          <t>roborock.krng.n</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C21" t="n">
-        <v>2368</v>
+        <v>3345</v>
       </c>
       <c r="D21" t="n">
+        <v>124</v>
+      </c>
+      <c r="E21" t="n">
         <v>18</v>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
       <c r="F21" t="n">
-        <v>0.76</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>longrobot_284</t>
+          <t>homesmediant99</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22" t="n">
-        <v>1593</v>
+        <v>917</v>
       </c>
       <c r="D22" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
-        <v>2.39</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>hatechz</t>
+          <t>longrobot_284</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>6</v>
       </c>
       <c r="C23" t="n">
-        <v>1351</v>
+        <v>1593</v>
       </c>
       <c r="D23" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>1.85</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>homesmediant99</t>
+          <t>hatechz</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>6</v>
       </c>
       <c r="C24" t="n">
-        <v>825</v>
+        <v>1351</v>
       </c>
       <c r="D24" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>2.67</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="25">
@@ -979,45 +979,45 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>tn.robot76</t>
+          <t>mi360vn</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>4</v>
       </c>
       <c r="C26" t="n">
-        <v>928</v>
+        <v>5975</v>
       </c>
       <c r="D26" t="n">
-        <v>19</v>
+        <v>598</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F26" t="n">
-        <v>2.16</v>
+        <v>10.51</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>mi360vn</t>
+          <t>tn.robot76</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C27" t="n">
-        <v>5844</v>
+        <v>928</v>
       </c>
       <c r="D27" t="n">
-        <v>595</v>
+        <v>19</v>
       </c>
       <c r="E27" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>10.69</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="28">
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>577</v>
+        <v>587</v>
       </c>
       <c r="C43" t="n">
-        <v>1077798</v>
+        <v>1081105</v>
       </c>
       <c r="D43" t="n">
-        <v>8471</v>
+        <v>8513</v>
       </c>
       <c r="E43" t="n">
         <v>1337</v>

</xml_diff>